<commit_message>
Update kasa standard cut length to 2.15m and unit to Boy
</commit_message>
<xml_diff>
--- a/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
+++ b/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
@@ -1106,17 +1106,17 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>140 mm Duvar</t>
+          <t>140 x 36 mm</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>4.95 kg/takım</t>
+          <t>4.95 kg/boy</t>
         </is>
       </c>
       <c r="F7" s="11" t="n">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="K7" s="16" t="inlineStr">
         <is>
-          <t>Saatte ~13 Takım</t>
+          <t>Saatte ~13 Boy</t>
         </is>
       </c>
       <c r="L7" s="11" t="n">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="N7" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~15 Takım</t>
+          <t>Saatte ~15 Boy</t>
         </is>
       </c>
       <c r="O7" s="18" t="n">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="T7" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~10 Takım</t>
+          <t>Saatte ~10 Boy</t>
         </is>
       </c>
       <c r="U7" s="20" t="n">
@@ -1206,17 +1206,17 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>100 mm Duvar</t>
+          <t>100 x 36 mm</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>4.00 kg/takım</t>
+          <t>4.00 kg/boy</t>
         </is>
       </c>
       <c r="F8" s="25" t="n">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="K8" s="30" t="inlineStr">
         <is>
-          <t>Saatte ~16 Takım</t>
+          <t>Saatte ~16 Boy</t>
         </is>
       </c>
       <c r="L8" s="25" t="n">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="N8" s="31" t="inlineStr">
         <is>
-          <t>Saatte ~17 Takım</t>
+          <t>Saatte ~17 Boy</t>
         </is>
       </c>
       <c r="O8" s="32" t="n">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="T8" s="31" t="inlineStr">
         <is>
-          <t>Saatte ~15 Takım</t>
+          <t>Saatte ~15 Boy</t>
         </is>
       </c>
       <c r="U8" s="34" t="n">
@@ -1412,17 +1412,17 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>200 mm Duvar</t>
+          <t>200 x 36 mm</t>
         </is>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
-          <t>6.66 kg/takım</t>
+          <t>6.66 kg/boy</t>
         </is>
       </c>
       <c r="F10" s="25" t="n">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="K10" s="30" t="inlineStr">
         <is>
-          <t>Saatte ~11 Takım</t>
+          <t>Saatte ~11 Boy</t>
         </is>
       </c>
       <c r="L10" s="25" t="n">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="N10" s="31" t="inlineStr">
         <is>
-          <t>Saatte ~13 Takım</t>
+          <t>Saatte ~13 Boy</t>
         </is>
       </c>
       <c r="O10" s="32" t="n">
@@ -5313,12 +5313,12 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>140 mm Duvar</t>
+          <t>140 x 36 mm</t>
         </is>
       </c>
       <c r="E8" s="52" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="J8" s="24" t="inlineStr">
         <is>
-          <t>4.95 kg/takım</t>
+          <t>4.95 kg/boy</t>
         </is>
       </c>
       <c r="K8" s="25" t="n">
@@ -5353,7 +5353,7 @@
       </c>
       <c r="M8" s="30" t="inlineStr">
         <is>
-          <t>Saatte ~13 Takım</t>
+          <t>Saatte ~13 Boy</t>
         </is>
       </c>
       <c r="N8" s="53" t="n">
@@ -5373,12 +5373,12 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>200 mm Duvar</t>
+          <t>200 x 36 mm</t>
         </is>
       </c>
       <c r="E9" s="54" t="inlineStr">
@@ -5402,7 +5402,7 @@
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>6.66 kg/takım</t>
+          <t>6.66 kg/boy</t>
         </is>
       </c>
       <c r="K9" s="11" t="n">
@@ -5413,7 +5413,7 @@
       </c>
       <c r="M9" s="16" t="inlineStr">
         <is>
-          <t>Saatte ~11 Takım</t>
+          <t>Saatte ~11 Boy</t>
         </is>
       </c>
       <c r="N9" s="55" t="n">
@@ -5493,12 +5493,12 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>100 mm Duvar</t>
+          <t>100 x 36 mm</t>
         </is>
       </c>
       <c r="E11" s="54" t="inlineStr">
@@ -5522,7 +5522,7 @@
       </c>
       <c r="J11" s="10" t="inlineStr">
         <is>
-          <t>4.00 kg/takım</t>
+          <t>4.00 kg/boy</t>
         </is>
       </c>
       <c r="K11" s="11" t="n">
@@ -5533,7 +5533,7 @@
       </c>
       <c r="M11" s="16" t="inlineStr">
         <is>
-          <t>Saatte ~15 Takım</t>
+          <t>Saatte ~15 Boy</t>
         </is>
       </c>
       <c r="N11" s="55" t="n">
@@ -5553,12 +5553,12 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D12" s="23" t="inlineStr">
         <is>
-          <t>100 mm Duvar</t>
+          <t>100 x 36 mm</t>
         </is>
       </c>
       <c r="E12" s="52" t="inlineStr">
@@ -5582,7 +5582,7 @@
       </c>
       <c r="J12" s="24" t="inlineStr">
         <is>
-          <t>4.00 kg/takım</t>
+          <t>4.00 kg/boy</t>
         </is>
       </c>
       <c r="K12" s="25" t="n">
@@ -5593,7 +5593,7 @@
       </c>
       <c r="M12" s="30" t="inlineStr">
         <is>
-          <t>Saatte ~16 Takım</t>
+          <t>Saatte ~16 Boy</t>
         </is>
       </c>
       <c r="N12" s="53" t="n">
@@ -5613,12 +5613,12 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>140 mm Duvar</t>
+          <t>140 x 36 mm</t>
         </is>
       </c>
       <c r="E13" s="54" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>4.95 kg/takım</t>
+          <t>4.95 kg/boy</t>
         </is>
       </c>
       <c r="K13" s="11" t="n">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="M13" s="16" t="inlineStr">
         <is>
-          <t>Saatte ~14 Takım</t>
+          <t>Saatte ~14 Boy</t>
         </is>
       </c>
       <c r="N13" s="55" t="n">
@@ -6033,12 +6033,12 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
         <is>
-          <t>140 mm Duvar</t>
+          <t>140 x 36 mm</t>
         </is>
       </c>
       <c r="E20" s="52" t="inlineStr">
@@ -6062,7 +6062,7 @@
       </c>
       <c r="J20" s="24" t="inlineStr">
         <is>
-          <t>4.95 kg/takım</t>
+          <t>4.95 kg/boy</t>
         </is>
       </c>
       <c r="K20" s="25" t="n">
@@ -6073,7 +6073,7 @@
       </c>
       <c r="M20" s="30" t="inlineStr">
         <is>
-          <t>Saatte ~10 Takım</t>
+          <t>Saatte ~10 Boy</t>
         </is>
       </c>
       <c r="N20" s="53" t="n">
@@ -6693,12 +6693,12 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
         <is>
-          <t>200 mm Duvar</t>
+          <t>200 x 36 mm</t>
         </is>
       </c>
       <c r="E31" s="54" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="J31" s="10" t="inlineStr">
         <is>
-          <t>6.66 kg/takım</t>
+          <t>6.66 kg/boy</t>
         </is>
       </c>
       <c r="K31" s="11" t="n">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="M31" s="16" t="inlineStr">
         <is>
-          <t>Saatte ~20 Takım</t>
+          <t>Saatte ~20 Boy</t>
         </is>
       </c>
       <c r="N31" s="55" t="n">
@@ -6873,12 +6873,12 @@
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D34" s="23" t="inlineStr">
         <is>
-          <t>200 mm Duvar</t>
+          <t>200 x 36 mm</t>
         </is>
       </c>
       <c r="E34" s="52" t="inlineStr">
@@ -6902,7 +6902,7 @@
       </c>
       <c r="J34" s="24" t="inlineStr">
         <is>
-          <t>6.66 kg/takım</t>
+          <t>6.66 kg/boy</t>
         </is>
       </c>
       <c r="K34" s="25" t="n">
@@ -6913,7 +6913,7 @@
       </c>
       <c r="M34" s="30" t="inlineStr">
         <is>
-          <t>Saatte ~14 Takım</t>
+          <t>Saatte ~14 Boy</t>
         </is>
       </c>
       <c r="N34" s="53" t="n">
@@ -7113,12 +7113,12 @@
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D38" s="23" t="inlineStr">
         <is>
-          <t>140 mm Duvar</t>
+          <t>140 x 36 mm</t>
         </is>
       </c>
       <c r="E38" s="52" t="inlineStr">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="J38" s="24" t="inlineStr">
         <is>
-          <t>4.95 kg/takım</t>
+          <t>4.95 kg/boy</t>
         </is>
       </c>
       <c r="K38" s="25" t="n">
@@ -7153,7 +7153,7 @@
       </c>
       <c r="M38" s="30" t="inlineStr">
         <is>
-          <t>Saatte ~6 Takım</t>
+          <t>Saatte ~6 Boy</t>
         </is>
       </c>
       <c r="N38" s="53" t="n">
@@ -7173,12 +7173,12 @@
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>140 mm Duvar</t>
+          <t>140 x 36 mm</t>
         </is>
       </c>
       <c r="E39" s="54" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="J39" s="10" t="inlineStr">
         <is>
-          <t>4.95 kg/takım</t>
+          <t>4.95 kg/boy</t>
         </is>
       </c>
       <c r="K39" s="11" t="n">
@@ -7213,7 +7213,7 @@
       </c>
       <c r="M39" s="16" t="inlineStr">
         <is>
-          <t>Saatte ~17 Takım</t>
+          <t>Saatte ~17 Boy</t>
         </is>
       </c>
       <c r="N39" s="55" t="n">
@@ -7233,12 +7233,12 @@
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D40" s="23" t="inlineStr">
         <is>
-          <t>100 mm Duvar</t>
+          <t>100 x 36 mm</t>
         </is>
       </c>
       <c r="E40" s="52" t="inlineStr">
@@ -7262,7 +7262,7 @@
       </c>
       <c r="J40" s="24" t="inlineStr">
         <is>
-          <t>4.00 kg/takım</t>
+          <t>4.00 kg/boy</t>
         </is>
       </c>
       <c r="K40" s="25" t="n">
@@ -7273,7 +7273,7 @@
       </c>
       <c r="M40" s="30" t="inlineStr">
         <is>
-          <t>Saatte ~14 Takım</t>
+          <t>Saatte ~14 Boy</t>
         </is>
       </c>
       <c r="N40" s="53" t="n">
@@ -7293,12 +7293,12 @@
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>2.20 m Yan + 1.05 m Üst (Takım)</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
         <is>
-          <t>100 mm Duvar</t>
+          <t>100 x 36 mm</t>
         </is>
       </c>
       <c r="E41" s="54" t="inlineStr">
@@ -7322,7 +7322,7 @@
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>4.00 kg/takım</t>
+          <t>4.00 kg/boy</t>
         </is>
       </c>
       <c r="K41" s="11" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="M41" s="16" t="inlineStr">
         <is>
-          <t>Saatte ~14 Takım</t>
+          <t>Saatte ~14 Boy</t>
         </is>
       </c>
       <c r="N41" s="55" t="n">

</xml_diff>

<commit_message>
Remove 0 kg phantom rows (duplicate Dişbudak and Seren Cift Kafa)
</commit_message>
<xml_diff>
--- a/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
+++ b/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
@@ -292,18 +292,6 @@
     <xf numFmtId="165" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -321,6 +309,18 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="4" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -701,7 +701,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X33"/>
+  <dimension ref="A1:X31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1296,7 +1296,7 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>DIŞBUDAK Levha</t>
+          <t>DİŞBUDAK Levha</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -3619,251 +3619,41 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>DİŞBUDAK Levha</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>WPC Levha Plaka</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>207 cm (2.07 m)</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>En: 94 cm (2 mm)</t>
-        </is>
-      </c>
-      <c r="E31" s="10" t="inlineStr">
-        <is>
-          <t>4.77 kg/plaka</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="12" t="inlineStr">
-        <is>
-          <t>Hat 201</t>
-        </is>
-      </c>
-      <c r="H31" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L31" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" s="13" t="n">
-        <v>187.9</v>
-      </c>
-      <c r="N31" s="17" t="inlineStr">
-        <is>
-          <t>Saatte ~39 Plaka</t>
-        </is>
-      </c>
-      <c r="O31" s="39" t="n">
-        <v>0</v>
-      </c>
-      <c r="P31" s="17" t="inlineStr">
-        <is>
-          <t>KLP-201</t>
-        </is>
-      </c>
-      <c r="Q31" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R31" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S31" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T31" s="17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="U31" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="V31" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W31" s="14" t="n">
-        <v>90</v>
-      </c>
-      <c r="X31" s="8" t="inlineStr">
-        <is>
-          <t>Levha Özel Hattı (Hat 201)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="22" t="inlineStr">
-        <is>
-          <t>SEREN (Çift Kafa)</t>
-        </is>
-      </c>
-      <c r="B32" s="23" t="inlineStr">
-        <is>
-          <t>Seren Çıtası</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
-        <is>
-          <t>2.10 Metre</t>
-        </is>
-      </c>
-      <c r="D32" s="23" t="inlineStr">
-        <is>
-          <t>38 x 45 mm</t>
-        </is>
-      </c>
-      <c r="E32" s="24" t="inlineStr">
-        <is>
-          <t>3.39 kg/boy</t>
-        </is>
-      </c>
-      <c r="F32" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="26" t="inlineStr">
-        <is>
-          <t>Hat 104</t>
-        </is>
-      </c>
-      <c r="H32" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I32" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" s="40" t="n">
-        <v>0</v>
-      </c>
-      <c r="K32" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="L32" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" s="27" t="n">
-        <v>99.2</v>
-      </c>
-      <c r="N32" s="31" t="inlineStr">
-        <is>
-          <t>Saatte ~29 Boy</t>
-        </is>
-      </c>
-      <c r="O32" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="P32" s="31" t="inlineStr">
-        <is>
-          <t>KLP-104</t>
-        </is>
-      </c>
-      <c r="Q32" s="33" t="inlineStr">
-        <is>
-          <t>Hat 105</t>
-        </is>
-      </c>
-      <c r="R32" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S32" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T32" s="31" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="U32" s="34" t="n">
-        <v>92.2</v>
-      </c>
-      <c r="V32" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="W32" s="28" t="n">
-        <v>45</v>
-      </c>
-      <c r="X32" s="23" t="inlineStr">
-        <is>
-          <t>Standart Planlama</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="42" t="inlineStr">
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="38" t="inlineStr">
         <is>
           <t>GENEL TOPLAM / FABRİKA</t>
         </is>
       </c>
-      <c r="B33" s="43" t="n"/>
-      <c r="C33" s="43" t="n"/>
-      <c r="D33" s="43" t="n"/>
-      <c r="E33" s="43" t="n"/>
-      <c r="F33" s="44" t="n">
+      <c r="B31" s="39" t="n"/>
+      <c r="C31" s="39" t="n"/>
+      <c r="D31" s="39" t="n"/>
+      <c r="E31" s="39" t="n"/>
+      <c r="F31" s="40" t="n">
         <v>1237183.51</v>
       </c>
-      <c r="G33" s="43" t="n"/>
-      <c r="H33" s="45" t="n">
+      <c r="G31" s="39" t="n"/>
+      <c r="H31" s="41" t="n">
         <v>11580</v>
       </c>
-      <c r="I33" s="43" t="n"/>
-      <c r="J33" s="43" t="n"/>
-      <c r="K33" s="43" t="n"/>
-      <c r="L33" s="43" t="n"/>
-      <c r="M33" s="43" t="n"/>
-      <c r="N33" s="43" t="n"/>
-      <c r="O33" s="43" t="n"/>
-      <c r="P33" s="43" t="n"/>
-      <c r="Q33" s="43" t="n"/>
-      <c r="R33" s="45" t="n">
+      <c r="I31" s="39" t="n"/>
+      <c r="J31" s="39" t="n"/>
+      <c r="K31" s="39" t="n"/>
+      <c r="L31" s="39" t="n"/>
+      <c r="M31" s="39" t="n"/>
+      <c r="N31" s="39" t="n"/>
+      <c r="O31" s="39" t="n"/>
+      <c r="P31" s="39" t="n"/>
+      <c r="Q31" s="39" t="n"/>
+      <c r="R31" s="41" t="n">
         <v>4908</v>
       </c>
-      <c r="S33" s="43" t="n"/>
-      <c r="T33" s="43" t="n"/>
-      <c r="U33" s="43" t="n"/>
-      <c r="V33" s="43" t="n"/>
-      <c r="W33" s="43" t="n"/>
-      <c r="X33" s="43" t="n"/>
+      <c r="S31" s="39" t="n"/>
+      <c r="T31" s="39" t="n"/>
+      <c r="U31" s="39" t="n"/>
+      <c r="V31" s="39" t="n"/>
+      <c r="W31" s="39" t="n"/>
+      <c r="X31" s="39" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3992,7 +3782,7 @@
       <c r="E4" s="25" t="n">
         <v>33263.65</v>
       </c>
-      <c r="F4" s="46" t="n">
+      <c r="F4" s="42" t="n">
         <v>33.26</v>
       </c>
       <c r="G4" s="29" t="n">
@@ -4007,7 +3797,7 @@
       <c r="J4" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="K4" s="47" t="inlineStr">
+      <c r="K4" s="43" t="inlineStr">
         <is>
           <t>35X100 PERVAZ, 35X150 PERVAZ, 35X80 PERVAZ</t>
         </is>
@@ -4033,7 +3823,7 @@
       <c r="E5" s="11" t="n">
         <v>91560.17999999998</v>
       </c>
-      <c r="F5" s="48" t="n">
+      <c r="F5" s="44" t="n">
         <v>91.56</v>
       </c>
       <c r="G5" s="15" t="n">
@@ -4048,7 +3838,7 @@
       <c r="J5" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K5" s="49" t="inlineStr">
+      <c r="K5" s="45" t="inlineStr">
         <is>
           <t>100 mm KASA, 140 mm KASA, CAM ÇITASI</t>
         </is>
@@ -4074,7 +3864,7 @@
       <c r="E6" s="25" t="n">
         <v>69803</v>
       </c>
-      <c r="F6" s="46" t="n">
+      <c r="F6" s="42" t="n">
         <v>69.8</v>
       </c>
       <c r="G6" s="29" t="n">
@@ -4089,7 +3879,7 @@
       <c r="J6" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="K6" s="47" t="inlineStr">
+      <c r="K6" s="43" t="inlineStr">
         <is>
           <t>50X80 PERVAZ, SEREN</t>
         </is>
@@ -4115,7 +3905,7 @@
       <c r="E7" s="11" t="n">
         <v>154861.98</v>
       </c>
-      <c r="F7" s="48" t="n">
+      <c r="F7" s="44" t="n">
         <v>154.86</v>
       </c>
       <c r="G7" s="15" t="n">
@@ -4130,7 +3920,7 @@
       <c r="J7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="K7" s="49" t="inlineStr">
+      <c r="K7" s="45" t="inlineStr">
         <is>
           <t>SEREN</t>
         </is>
@@ -4156,7 +3946,7 @@
       <c r="E8" s="25" t="n">
         <v>137071.86</v>
       </c>
-      <c r="F8" s="46" t="n">
+      <c r="F8" s="42" t="n">
         <v>137.07</v>
       </c>
       <c r="G8" s="29" t="n">
@@ -4171,7 +3961,7 @@
       <c r="J8" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="K8" s="47" t="inlineStr">
+      <c r="K8" s="43" t="inlineStr">
         <is>
           <t>140 mm KASA, SEREN</t>
         </is>
@@ -4197,7 +3987,7 @@
       <c r="E9" s="11" t="n">
         <v>112898.9699999999</v>
       </c>
-      <c r="F9" s="48" t="n">
+      <c r="F9" s="44" t="n">
         <v>112.9</v>
       </c>
       <c r="G9" s="15" t="n">
@@ -4212,7 +4002,7 @@
       <c r="J9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="K9" s="49" t="inlineStr">
+      <c r="K9" s="45" t="inlineStr">
         <is>
           <t>100 mm KASA, 140 mm KASA, 200 mm KASA</t>
         </is>
@@ -4238,7 +4028,7 @@
       <c r="E10" s="25" t="n">
         <v>135361.61</v>
       </c>
-      <c r="F10" s="46" t="n">
+      <c r="F10" s="42" t="n">
         <v>135.36</v>
       </c>
       <c r="G10" s="29" t="n">
@@ -4253,7 +4043,7 @@
       <c r="J10" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="K10" s="47" t="inlineStr">
+      <c r="K10" s="43" t="inlineStr">
         <is>
           <t>100 mm KASA, 140 mm KASA, 200 mm KASA</t>
         </is>
@@ -4279,7 +4069,7 @@
       <c r="E11" s="11" t="n">
         <v>109257.63</v>
       </c>
-      <c r="F11" s="48" t="n">
+      <c r="F11" s="44" t="n">
         <v>109.26</v>
       </c>
       <c r="G11" s="15" t="n">
@@ -4294,7 +4084,7 @@
       <c r="J11" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="K11" s="49" t="inlineStr">
+      <c r="K11" s="45" t="inlineStr">
         <is>
           <t>100 mm KASA, 140 mm KASA, 200 mm KASA</t>
         </is>
@@ -4320,7 +4110,7 @@
       <c r="E12" s="25" t="n">
         <v>118327.55</v>
       </c>
-      <c r="F12" s="46" t="n">
+      <c r="F12" s="42" t="n">
         <v>118.33</v>
       </c>
       <c r="G12" s="29" t="n">
@@ -4335,7 +4125,7 @@
       <c r="J12" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="K12" s="47" t="inlineStr">
+      <c r="K12" s="43" t="inlineStr">
         <is>
           <t>50X80 PERVAZ, 80X80 PERVAZ</t>
         </is>
@@ -4361,7 +4151,7 @@
       <c r="E13" s="11" t="n">
         <v>274777.0800000001</v>
       </c>
-      <c r="F13" s="48" t="n">
+      <c r="F13" s="44" t="n">
         <v>274.78</v>
       </c>
       <c r="G13" s="15" t="n">
@@ -4376,7 +4166,7 @@
       <c r="J13" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="K13" s="49" t="inlineStr">
+      <c r="K13" s="45" t="inlineStr">
         <is>
           <t>ANTRASİT Levha, AY GRİ Levha, BEYAZ TEAK Levha</t>
         </is>
@@ -4402,22 +4192,22 @@
       <c r="E14" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="40" t="n">
+      <c r="F14" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="46" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="34" t="n">
         <v>250</v>
       </c>
-      <c r="I14" s="41" t="n">
+      <c r="I14" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="47" t="inlineStr">
+      <c r="K14" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4443,22 +4233,22 @@
       <c r="E15" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="38" t="n">
+      <c r="F15" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="48" t="n">
         <v>0</v>
       </c>
       <c r="H15" s="20" t="n">
         <v>250</v>
       </c>
-      <c r="I15" s="39" t="n">
+      <c r="I15" s="49" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="49" t="inlineStr">
+      <c r="K15" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4484,22 +4274,22 @@
       <c r="E16" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="40" t="n">
+      <c r="F16" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="46" t="n">
         <v>0</v>
       </c>
       <c r="H16" s="34" t="n">
         <v>250</v>
       </c>
-      <c r="I16" s="41" t="n">
+      <c r="I16" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J16" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="47" t="inlineStr">
+      <c r="K16" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4525,22 +4315,22 @@
       <c r="E17" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="38" t="n">
+      <c r="F17" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="48" t="n">
         <v>0</v>
       </c>
       <c r="H17" s="20" t="n">
         <v>250</v>
       </c>
-      <c r="I17" s="39" t="n">
+      <c r="I17" s="49" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="49" t="inlineStr">
+      <c r="K17" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4566,22 +4356,22 @@
       <c r="E18" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="40" t="n">
+      <c r="F18" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="46" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="34" t="n">
         <v>180</v>
       </c>
-      <c r="I18" s="41" t="n">
+      <c r="I18" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K18" s="47" t="inlineStr">
+      <c r="K18" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4607,22 +4397,22 @@
       <c r="E19" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="38" t="n">
+      <c r="F19" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="48" t="n">
         <v>0</v>
       </c>
       <c r="H19" s="20" t="n">
         <v>180</v>
       </c>
-      <c r="I19" s="39" t="n">
+      <c r="I19" s="49" t="n">
         <v>0</v>
       </c>
       <c r="J19" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="49" t="inlineStr">
+      <c r="K19" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4648,22 +4438,22 @@
       <c r="E20" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="40" t="n">
+      <c r="F20" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="46" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="34" t="n">
         <v>180</v>
       </c>
-      <c r="I20" s="41" t="n">
+      <c r="I20" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="47" t="inlineStr">
+      <c r="K20" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4689,22 +4479,22 @@
       <c r="E21" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="38" t="n">
+      <c r="F21" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="48" t="n">
         <v>0</v>
       </c>
       <c r="H21" s="20" t="n">
         <v>180</v>
       </c>
-      <c r="I21" s="39" t="n">
+      <c r="I21" s="49" t="n">
         <v>0</v>
       </c>
       <c r="J21" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K21" s="49" t="inlineStr">
+      <c r="K21" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4730,22 +4520,22 @@
       <c r="E22" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="F22" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="40" t="n">
+      <c r="F22" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="46" t="n">
         <v>0</v>
       </c>
       <c r="H22" s="34" t="n">
         <v>180</v>
       </c>
-      <c r="I22" s="41" t="n">
+      <c r="I22" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J22" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="47" t="inlineStr">
+      <c r="K22" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4771,22 +4561,22 @@
       <c r="E23" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="38" t="n">
+      <c r="F23" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="48" t="n">
         <v>0</v>
       </c>
       <c r="H23" s="20" t="n">
         <v>180</v>
       </c>
-      <c r="I23" s="39" t="n">
+      <c r="I23" s="49" t="n">
         <v>0</v>
       </c>
       <c r="J23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="49" t="inlineStr">
+      <c r="K23" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4812,22 +4602,22 @@
       <c r="E24" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="F24" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="40" t="n">
+      <c r="F24" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="46" t="n">
         <v>0</v>
       </c>
       <c r="H24" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="I24" s="41" t="n">
+      <c r="I24" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J24" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="47" t="inlineStr">
+      <c r="K24" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4853,22 +4643,22 @@
       <c r="E25" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="38" t="n">
+      <c r="F25" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="48" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="20" t="n">
         <v>400</v>
       </c>
-      <c r="I25" s="39" t="n">
+      <c r="I25" s="49" t="n">
         <v>0</v>
       </c>
       <c r="J25" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="49" t="inlineStr">
+      <c r="K25" s="45" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4894,22 +4684,22 @@
       <c r="E26" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="F26" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="40" t="n">
+      <c r="F26" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="46" t="n">
         <v>0</v>
       </c>
       <c r="H26" s="34" t="n">
         <v>400</v>
       </c>
-      <c r="I26" s="41" t="n">
+      <c r="I26" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J26" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="47" t="inlineStr">
+      <c r="K26" s="43" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4921,24 +4711,24 @@
           <t>GENEL MAKİNE TOPLAMI</t>
         </is>
       </c>
-      <c r="B27" s="43" t="n"/>
-      <c r="C27" s="45" t="n">
+      <c r="B27" s="39" t="n"/>
+      <c r="C27" s="41" t="n">
         <v>17304</v>
       </c>
-      <c r="D27" s="44" t="n">
+      <c r="D27" s="40" t="n">
         <v>1442</v>
       </c>
-      <c r="E27" s="44" t="n">
+      <c r="E27" s="40" t="n">
         <v>1237183.51</v>
       </c>
       <c r="F27" s="51" t="n">
         <v>1237.18</v>
       </c>
-      <c r="G27" s="43" t="n"/>
-      <c r="H27" s="43" t="n"/>
-      <c r="I27" s="43" t="n"/>
-      <c r="J27" s="43" t="n"/>
-      <c r="K27" s="43" t="n"/>
+      <c r="G27" s="39" t="n"/>
+      <c r="H27" s="39" t="n"/>
+      <c r="I27" s="39" t="n"/>
+      <c r="J27" s="39" t="n"/>
+      <c r="K27" s="39" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5183,7 +4973,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
         <is>
-          <t>DIŞBUDAK Levha</t>
+          <t>DİŞBUDAK Levha</t>
         </is>
       </c>
       <c r="B6" s="23" t="inlineStr">
@@ -7466,25 +7256,25 @@
           <t>GENEL TOPLAM</t>
         </is>
       </c>
-      <c r="B44" s="43" t="n"/>
-      <c r="C44" s="43" t="n"/>
-      <c r="D44" s="43" t="n"/>
-      <c r="E44" s="43" t="n"/>
-      <c r="F44" s="43" t="n"/>
-      <c r="G44" s="45" t="n">
+      <c r="B44" s="39" t="n"/>
+      <c r="C44" s="39" t="n"/>
+      <c r="D44" s="39" t="n"/>
+      <c r="E44" s="39" t="n"/>
+      <c r="F44" s="39" t="n"/>
+      <c r="G44" s="41" t="n">
         <v>17304</v>
       </c>
-      <c r="H44" s="43" t="n"/>
-      <c r="I44" s="44" t="n">
+      <c r="H44" s="39" t="n"/>
+      <c r="I44" s="40" t="n">
         <v>379264</v>
       </c>
-      <c r="J44" s="43" t="n"/>
-      <c r="K44" s="44" t="n">
+      <c r="J44" s="39" t="n"/>
+      <c r="K44" s="40" t="n">
         <v>1237183.51</v>
       </c>
-      <c r="L44" s="43" t="n"/>
-      <c r="M44" s="43" t="n"/>
-      <c r="N44" s="43" t="n"/>
+      <c r="L44" s="39" t="n"/>
+      <c r="M44" s="39" t="n"/>
+      <c r="N44" s="39" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Fix Ana Rota assignment using actual top production hat and resolve 148.8% anomaly
</commit_message>
<xml_diff>
--- a/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
+++ b/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
@@ -981,7 +981,7 @@
       </c>
       <c r="V5" s="21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Hat 107</t>
         </is>
       </c>
       <c r="W5" s="14" t="n">
@@ -1162,18 +1162,18 @@
       </c>
       <c r="Q7" s="19" t="inlineStr">
         <is>
-          <t>Hat 102</t>
+          <t>Hat 108</t>
         </is>
       </c>
       <c r="R7" s="20" t="n">
-        <v>312</v>
+        <v>636</v>
       </c>
       <c r="S7" s="20" t="n">
-        <v>49.8</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="T7" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~10 Boy</t>
+          <t>Saatte ~14 Boy</t>
         </is>
       </c>
       <c r="U7" s="20" t="n">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="V7" s="21" t="inlineStr">
         <is>
-          <t>Hat 108</t>
+          <t>Hat 102</t>
         </is>
       </c>
       <c r="W7" s="14" t="n">
@@ -1224,68 +1224,68 @@
       </c>
       <c r="G8" s="26" t="inlineStr">
         <is>
+          <t>Hat 102</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="n">
+        <v>1140</v>
+      </c>
+      <c r="I8" s="28" t="n">
+        <v>95</v>
+      </c>
+      <c r="J8" s="29" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="K8" s="30" t="inlineStr">
+        <is>
+          <t>Saatte ~15 Boy</t>
+        </is>
+      </c>
+      <c r="L8" s="25" t="n">
+        <v>1408.8</v>
+      </c>
+      <c r="M8" s="27" t="n">
+        <v>63</v>
+      </c>
+      <c r="N8" s="31" t="inlineStr">
+        <is>
+          <t>Saatte ~16 Boy</t>
+        </is>
+      </c>
+      <c r="O8" s="32" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="P8" s="31" t="inlineStr">
+        <is>
+          <t>KLP-102</t>
+        </is>
+      </c>
+      <c r="Q8" s="33" t="inlineStr">
+        <is>
           <t>Hat 108</t>
         </is>
       </c>
-      <c r="H8" s="27" t="n">
+      <c r="R8" s="34" t="n">
         <v>1008</v>
       </c>
-      <c r="I8" s="28" t="n">
-        <v>84</v>
-      </c>
-      <c r="J8" s="29" t="n">
+      <c r="S8" s="34" t="n">
         <v>63.6</v>
       </c>
-      <c r="K8" s="30" t="inlineStr">
+      <c r="T8" s="31" t="inlineStr">
         <is>
           <t>Saatte ~16 Boy</t>
         </is>
       </c>
-      <c r="L8" s="25" t="n">
-        <v>1526.4</v>
-      </c>
-      <c r="M8" s="27" t="n">
+      <c r="U8" s="34" t="n">
         <v>69.5</v>
       </c>
-      <c r="N8" s="31" t="inlineStr">
-        <is>
-          <t>Saatte ~17 Boy</t>
-        </is>
-      </c>
-      <c r="O8" s="32" t="n">
-        <v>0.915</v>
-      </c>
-      <c r="P8" s="31" t="inlineStr">
-        <is>
-          <t>KLP-106</t>
-        </is>
-      </c>
-      <c r="Q8" s="33" t="inlineStr">
-        <is>
-          <t>Hat 102</t>
-        </is>
-      </c>
-      <c r="R8" s="34" t="n">
-        <v>1140</v>
-      </c>
-      <c r="S8" s="34" t="n">
-        <v>58.7</v>
-      </c>
-      <c r="T8" s="31" t="inlineStr">
-        <is>
-          <t>Saatte ~15 Boy</t>
-        </is>
-      </c>
-      <c r="U8" s="34" t="n">
-        <v>63</v>
-      </c>
       <c r="V8" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Hat 107</t>
         </is>
       </c>
       <c r="W8" s="28" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="X8" s="23" t="inlineStr">
         <is>
@@ -1466,34 +1466,28 @@
           <t>KLP-107</t>
         </is>
       </c>
-      <c r="Q10" s="35" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="R10" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="S10" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="Q10" s="33" t="inlineStr">
+        <is>
+          <t>Hat 106</t>
+        </is>
+      </c>
+      <c r="R10" s="34" t="n">
+        <v>24</v>
+      </c>
+      <c r="S10" s="34" t="n">
+        <v>136.5</v>
       </c>
       <c r="T10" s="31" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="U10" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Saatte ~20 Boy</t>
+        </is>
+      </c>
+      <c r="U10" s="34" t="n">
+        <v>76.14</v>
       </c>
       <c r="V10" s="35" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Hat 108</t>
         </is>
       </c>
       <c r="W10" s="28" t="n">
@@ -1501,7 +1495,7 @@
       </c>
       <c r="X10" s="23" t="inlineStr">
         <is>
-          <t>Tek Hat Kalıp Atamalı</t>
+          <t>Aktif Çift Hatlı Üretim (Yüksek Hacimli)</t>
         </is>
       </c>
     </row>
@@ -2172,68 +2166,68 @@
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
+          <t>Hat 101</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>324</v>
+      </c>
+      <c r="I17" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="J17" s="15" t="n">
+        <v>39.6</v>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Saatte ~18 Boy</t>
+        </is>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>950.4</v>
+      </c>
+      <c r="M17" s="13" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="N17" s="17" t="inlineStr">
+        <is>
+          <t>Saatte ~21 Boy</t>
+        </is>
+      </c>
+      <c r="O17" s="18" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="P17" s="17" t="inlineStr">
+        <is>
+          <t>KLP-101</t>
+        </is>
+      </c>
+      <c r="Q17" s="19" t="inlineStr">
+        <is>
           <t>Hat 109</t>
         </is>
       </c>
-      <c r="H17" s="13" t="n">
+      <c r="R17" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="I17" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="15" t="n">
+      <c r="S17" s="20" t="n">
         <v>126.5</v>
       </c>
-      <c r="K17" s="16" t="inlineStr">
+      <c r="T17" s="17" t="inlineStr">
         <is>
           <t>Saatte ~58 Boy</t>
         </is>
       </c>
-      <c r="L17" s="11" t="n">
-        <v>3036</v>
-      </c>
-      <c r="M17" s="13" t="n">
+      <c r="U17" s="20" t="n">
         <v>85</v>
       </c>
-      <c r="N17" s="17" t="inlineStr">
-        <is>
-          <t>Saatte ~39 Boy</t>
-        </is>
-      </c>
-      <c r="O17" s="18" t="n">
-        <v>1.488</v>
-      </c>
-      <c r="P17" s="17" t="inlineStr">
-        <is>
-          <t>KLP-103</t>
-        </is>
-      </c>
-      <c r="Q17" s="19" t="inlineStr">
-        <is>
-          <t>Hat 101</t>
-        </is>
-      </c>
-      <c r="R17" s="20" t="n">
-        <v>324</v>
-      </c>
-      <c r="S17" s="20" t="n">
-        <v>39.6</v>
-      </c>
-      <c r="T17" s="17" t="inlineStr">
-        <is>
-          <t>Saatte ~18 Boy</t>
-        </is>
-      </c>
-      <c r="U17" s="20" t="n">
-        <v>46.5</v>
-      </c>
       <c r="V17" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="W17" s="14" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="X17" s="8" t="inlineStr">
         <is>
@@ -3634,7 +3628,7 @@
       </c>
       <c r="G31" s="39" t="n"/>
       <c r="H31" s="41" t="n">
-        <v>11580</v>
+        <v>12024</v>
       </c>
       <c r="I31" s="39" t="n"/>
       <c r="J31" s="39" t="n"/>
@@ -3646,7 +3640,7 @@
       <c r="P31" s="39" t="n"/>
       <c r="Q31" s="39" t="n"/>
       <c r="R31" s="41" t="n">
-        <v>4908</v>
+        <v>4812</v>
       </c>
       <c r="S31" s="39" t="n"/>
       <c r="T31" s="39" t="n"/>

</xml_diff>

<commit_message>
feat(planlama): 26 urun katalogu, net kesim olculeri, acil oncelikleme ve siparis dondurma (preemption) ozellikleri eklendi
</commit_message>
<xml_diff>
--- a/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
+++ b/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
@@ -959,7 +959,7 @@
         </is>
       </c>
       <c r="F5" s="11" t="n">
-        <v>296887.79</v>
+        <v>298093.79</v>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
@@ -972,13 +972,13 @@
         </is>
       </c>
       <c r="I5" s="14" t="n">
-        <v>1598.4</v>
+        <v>1622.4</v>
       </c>
       <c r="J5" s="15" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="K5" s="16" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="L5" s="17" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         </is>
       </c>
       <c r="M5" s="11" t="n">
-        <v>2340</v>
+        <v>2323.2</v>
       </c>
       <c r="N5" s="14" t="n">
         <v>99.2</v>
@@ -997,7 +997,7 @@
         </is>
       </c>
       <c r="P5" s="19" t="n">
-        <v>0.983</v>
+        <v>0.976</v>
       </c>
       <c r="Q5" s="15" t="n">
         <v>45</v>
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="F6" s="26" t="n">
-        <v>185908.31</v>
+        <v>188073.31</v>
       </c>
       <c r="G6" s="27" t="inlineStr">
         <is>
@@ -1077,13 +1077,13 @@
         </is>
       </c>
       <c r="I6" s="28" t="n">
-        <v>1520.2</v>
+        <v>1538.2</v>
       </c>
       <c r="J6" s="29" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="K6" s="30" t="n">
-        <v>74.3</v>
+        <v>73.7</v>
       </c>
       <c r="L6" s="31" t="inlineStr">
         <is>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="M6" s="26" t="n">
-        <v>1783.2</v>
+        <v>1768.8</v>
       </c>
       <c r="N6" s="28" t="n">
         <v>73.59999999999999</v>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="P6" s="33" t="n">
-        <v>1.01</v>
+        <v>1.001</v>
       </c>
       <c r="Q6" s="29" t="n">
         <v>35</v>
@@ -1118,10 +1118,10 @@
         </is>
       </c>
       <c r="T6" s="35" t="n">
-        <v>1397</v>
+        <v>1421</v>
       </c>
       <c r="U6" s="35" t="n">
-        <v>52.3</v>
+        <v>52.6</v>
       </c>
       <c r="V6" s="32" t="inlineStr">
         <is>
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="F7" s="11" t="n">
-        <v>170210</v>
+        <v>172895</v>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
@@ -1182,21 +1182,21 @@
         </is>
       </c>
       <c r="I7" s="14" t="n">
-        <v>1561.3</v>
+        <v>1585.3</v>
       </c>
       <c r="J7" s="15" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K7" s="16" t="n">
-        <v>72</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="L7" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~14 Boy</t>
+          <t>Saatte ~15 Boy</t>
         </is>
       </c>
       <c r="M7" s="11" t="n">
-        <v>1728</v>
+        <v>1730.4</v>
       </c>
       <c r="N7" s="14" t="n">
         <v>74.09999999999999</v>
@@ -1207,7 +1207,7 @@
         </is>
       </c>
       <c r="P7" s="19" t="n">
-        <v>0.972</v>
+        <v>0.973</v>
       </c>
       <c r="Q7" s="15" t="n">
         <v>55</v>
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="F8" s="26" t="n">
-        <v>131789.8</v>
+        <v>132867.8</v>
       </c>
       <c r="G8" s="27" t="inlineStr">
         <is>
@@ -1328,10 +1328,10 @@
         </is>
       </c>
       <c r="T8" s="35" t="n">
-        <v>911</v>
+        <v>935</v>
       </c>
       <c r="U8" s="35" t="n">
-        <v>67.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="V8" s="32" t="inlineStr">
         <is>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="F9" s="11" t="n">
-        <v>118792.08</v>
+        <v>119746.08</v>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
@@ -1392,13 +1392,13 @@
         </is>
       </c>
       <c r="I9" s="14" t="n">
-        <v>1198.5</v>
+        <v>1204.5</v>
       </c>
       <c r="J9" s="15" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K9" s="16" t="n">
-        <v>99.09999999999999</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="L9" s="17" t="inlineStr">
         <is>
@@ -1406,7 +1406,7 @@
         </is>
       </c>
       <c r="M9" s="11" t="n">
-        <v>2378.4</v>
+        <v>2385.6</v>
       </c>
       <c r="N9" s="14" t="n">
         <v>187.9</v>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="P9" s="37" t="n">
-        <v>0.527</v>
+        <v>0.529</v>
       </c>
       <c r="Q9" s="15" t="n">
         <v>90</v>
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="F13" s="11" t="n">
-        <v>30621.25</v>
+        <v>32023.75</v>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
@@ -1830,13 +1830,13 @@
         </is>
       </c>
       <c r="I13" s="14" t="n">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="J13" s="15" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K13" s="16" t="n">
-        <v>92.5</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="L13" s="17" t="inlineStr">
         <is>
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="M13" s="11" t="n">
-        <v>2220</v>
+        <v>2253.6</v>
       </c>
       <c r="N13" s="14" t="n">
         <v>131.5</v>
@@ -1855,7 +1855,7 @@
         </is>
       </c>
       <c r="P13" s="37" t="n">
-        <v>0.703</v>
+        <v>0.7140000000000001</v>
       </c>
       <c r="Q13" s="15" t="n">
         <v>90</v>
@@ -1928,7 +1928,7 @@
         </is>
       </c>
       <c r="F14" s="26" t="n">
-        <v>27487</v>
+        <v>30342</v>
       </c>
       <c r="G14" s="27" t="inlineStr">
         <is>
@@ -1941,21 +1941,21 @@
         </is>
       </c>
       <c r="I14" s="28" t="n">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="J14" s="29" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K14" s="30" t="n">
-        <v>107.8</v>
+        <v>108.8</v>
       </c>
       <c r="L14" s="31" t="inlineStr">
         <is>
-          <t>Saatte ~28 Boy</t>
+          <t>Saatte ~29 Boy</t>
         </is>
       </c>
       <c r="M14" s="26" t="n">
-        <v>2587.2</v>
+        <v>2611.2</v>
       </c>
       <c r="N14" s="28" t="n">
         <v>96.09999999999999</v>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="P14" s="33" t="n">
-        <v>1.122</v>
+        <v>1.132</v>
       </c>
       <c r="Q14" s="29" t="n">
         <v>60</v>
@@ -3793,12 +3793,12 @@
       <c r="D31" s="40" t="n"/>
       <c r="E31" s="40" t="n"/>
       <c r="F31" s="41" t="n">
-        <v>1239963.98</v>
+        <v>1252309.48</v>
       </c>
       <c r="G31" s="40" t="n"/>
       <c r="H31" s="40" t="n"/>
       <c r="I31" s="42" t="n">
-        <v>10874.7</v>
+        <v>10980.7</v>
       </c>
       <c r="J31" s="40" t="n"/>
       <c r="K31" s="40" t="n"/>
@@ -3811,7 +3811,7 @@
       <c r="R31" s="40" t="n"/>
       <c r="S31" s="40" t="n"/>
       <c r="T31" s="42" t="n">
-        <v>4436.7</v>
+        <v>4484.7</v>
       </c>
       <c r="U31" s="40" t="n"/>
       <c r="V31" s="40" t="n"/>
@@ -3990,16 +3990,16 @@
         </is>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1539.1</v>
+        <v>1560.1</v>
       </c>
       <c r="E5" s="15" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>94501</v>
+        <v>95369</v>
       </c>
       <c r="G5" s="16" t="n">
-        <v>61.4</v>
+        <v>61.1</v>
       </c>
       <c r="H5" s="46" t="n">
         <v>4</v>
@@ -4037,16 +4037,16 @@
         </is>
       </c>
       <c r="D6" s="28" t="n">
-        <v>1409</v>
+        <v>1433</v>
       </c>
       <c r="E6" s="29" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>73771</v>
+        <v>75496</v>
       </c>
       <c r="G6" s="30" t="n">
-        <v>52.4</v>
+        <v>52.7</v>
       </c>
       <c r="H6" s="44" t="n">
         <v>2</v>
@@ -4084,16 +4084,16 @@
         </is>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1598.4</v>
+        <v>1622.4</v>
       </c>
       <c r="E7" s="15" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>155845.32</v>
+        <v>157051.32</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="H7" s="46" t="n">
         <v>1</v>
@@ -4178,16 +4178,16 @@
         </is>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1597.3</v>
+        <v>1621.3</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>115692</v>
+        <v>117509</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>72.40000000000001</v>
+        <v>72.5</v>
       </c>
       <c r="H9" s="46" t="n">
         <v>3</v>
@@ -4225,16 +4225,16 @@
         </is>
       </c>
       <c r="D10" s="28" t="n">
-        <v>1545.7</v>
+        <v>1569.7</v>
       </c>
       <c r="E10" s="29" t="n">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>138070</v>
+        <v>140925</v>
       </c>
       <c r="G10" s="30" t="n">
-        <v>89.3</v>
+        <v>89.8</v>
       </c>
       <c r="H10" s="44" t="n">
         <v>8</v>
@@ -4272,16 +4272,16 @@
         </is>
       </c>
       <c r="D11" s="14" t="n">
-        <v>1525.2</v>
+        <v>1549.2</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>102062.8</v>
+        <v>103140.8</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>66.90000000000001</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="H11" s="46" t="n">
         <v>3</v>
@@ -4319,16 +4319,16 @@
         </is>
       </c>
       <c r="D12" s="28" t="n">
-        <v>1532.2</v>
+        <v>1550.2</v>
       </c>
       <c r="E12" s="29" t="n">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F12" s="26" t="n">
-        <v>113918.31</v>
+        <v>114358.31</v>
       </c>
       <c r="G12" s="30" t="n">
-        <v>74.3</v>
+        <v>73.8</v>
       </c>
       <c r="H12" s="44" t="n">
         <v>2</v>
@@ -4366,23 +4366,23 @@
         </is>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2730.5</v>
+        <v>2746.5</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>274777.0800000001</v>
+        <v>277133.5800000001</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>100.6</v>
+        <v>100.9</v>
       </c>
       <c r="H13" s="46" t="n">
         <v>11</v>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
-          <t>Tek Göz (Geniş Düz Dudak)</t>
+          <t>Levha Kalıbı (Tek Kafa)</t>
         </is>
       </c>
       <c r="J13" s="8" t="inlineStr">
@@ -4405,16 +4405,16 @@
       <c r="B14" s="40" t="n"/>
       <c r="C14" s="40" t="n"/>
       <c r="D14" s="42" t="n">
-        <v>15736.4</v>
+        <v>15911.4</v>
       </c>
       <c r="E14" s="41" t="n">
-        <v>1444</v>
+        <v>1461</v>
       </c>
       <c r="F14" s="41" t="n">
-        <v>1239963.98</v>
+        <v>1252309.48</v>
       </c>
       <c r="G14" s="42" t="n">
-        <v>78.8</v>
+        <v>78.7</v>
       </c>
       <c r="H14" s="40" t="n"/>
       <c r="I14" s="40" t="n"/>
@@ -4584,13 +4584,13 @@
         </is>
       </c>
       <c r="H4" s="28" t="n">
-        <v>1598.4</v>
+        <v>1622.4</v>
       </c>
       <c r="I4" s="29" t="n">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="J4" s="29" t="n">
-        <v>45682</v>
+        <v>46047</v>
       </c>
       <c r="K4" s="25" t="inlineStr">
         <is>
@@ -4598,18 +4598,18 @@
         </is>
       </c>
       <c r="L4" s="26" t="n">
-        <v>155845.32</v>
+        <v>157051.32</v>
       </c>
       <c r="M4" s="30" t="n">
-        <v>97.5</v>
+        <v>96.8</v>
       </c>
       <c r="N4" s="31" t="inlineStr">
         <is>
-          <t>Saatte ~29 Boy</t>
+          <t>Saatte ~28 Boy</t>
         </is>
       </c>
       <c r="O4" s="48" t="n">
-        <v>0.5249300417507907</v>
+        <v>0.526852035394632</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -4674,7 +4674,7 @@
         </is>
       </c>
       <c r="O5" s="49" t="n">
-        <v>0.4607985730905269</v>
+        <v>0.4589343172831611</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -4714,13 +4714,13 @@
         </is>
       </c>
       <c r="H6" s="28" t="n">
-        <v>1198.5</v>
+        <v>1204.5</v>
       </c>
       <c r="I6" s="29" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J6" s="29" t="n">
-        <v>24904</v>
+        <v>25104</v>
       </c>
       <c r="K6" s="25" t="inlineStr">
         <is>
@@ -4728,10 +4728,10 @@
         </is>
       </c>
       <c r="L6" s="26" t="n">
-        <v>118792.08</v>
+        <v>119746.08</v>
       </c>
       <c r="M6" s="30" t="n">
-        <v>99.09999999999999</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="N6" s="31" t="inlineStr">
         <is>
@@ -4745,32 +4745,32 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>50X80 PERVAZ</t>
+          <t>140 mm KASA</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Pervaz Profili</t>
+          <t>Kasa Profili</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>2.20 Metre</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>50 x 80 mm</t>
+          <t>140 x 36 mm</t>
         </is>
       </c>
       <c r="E7" s="45" t="inlineStr">
         <is>
-          <t>Hat 109</t>
-        </is>
-      </c>
-      <c r="F7" s="13" t="inlineStr">
-        <is>
-          <t>Çift Göz (2 Kafa)</t>
+          <t>Hat 106</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>Tek Göz (1 Kafa)</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
@@ -4779,63 +4779,63 @@
         </is>
       </c>
       <c r="H7" s="14" t="n">
-        <v>1520.2</v>
+        <v>1585.3</v>
       </c>
       <c r="I7" s="15" t="n">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="J7" s="15" t="n">
-        <v>75361</v>
+        <v>22355</v>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>1.55 kg/boy</t>
+          <t>4.95 kg/boy</t>
         </is>
       </c>
       <c r="L7" s="11" t="n">
-        <v>112897.31</v>
+        <v>114247</v>
       </c>
       <c r="M7" s="16" t="n">
-        <v>74.3</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="N7" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~50 Boy</t>
+          <t>Saatte ~14 Boy</t>
         </is>
       </c>
       <c r="O7" s="49" t="n">
-        <v>0.6072741449803938</v>
+        <v>0.6607883397437752</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="23" t="inlineStr">
         <is>
-          <t>140 mm KASA</t>
+          <t>50X80 PERVAZ</t>
         </is>
       </c>
       <c r="B8" s="24" t="inlineStr">
         <is>
-          <t>Kasa Profili</t>
+          <t>Pervaz Profili</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>2.15 Metre (215 cm)</t>
+          <t>2.20 Metre</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>140 x 36 mm</t>
+          <t>50 x 80 mm</t>
         </is>
       </c>
       <c r="E8" s="43" t="inlineStr">
         <is>
-          <t>Hat 106</t>
-        </is>
-      </c>
-      <c r="F8" s="32" t="inlineStr">
-        <is>
-          <t>Tek Göz (1 Kafa)</t>
+          <t>Hat 109</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Çift Göz (2 Kafa)</t>
         </is>
       </c>
       <c r="G8" s="27" t="inlineStr">
@@ -4844,32 +4844,32 @@
         </is>
       </c>
       <c r="H8" s="28" t="n">
-        <v>1561.3</v>
+        <v>1538.2</v>
       </c>
       <c r="I8" s="29" t="n">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="J8" s="29" t="n">
-        <v>22015</v>
+        <v>75716</v>
       </c>
       <c r="K8" s="25" t="inlineStr">
         <is>
-          <t>4.95 kg/boy</t>
+          <t>1.55 kg/boy</t>
         </is>
       </c>
       <c r="L8" s="26" t="n">
-        <v>112430</v>
+        <v>113337.31</v>
       </c>
       <c r="M8" s="30" t="n">
-        <v>72</v>
+        <v>73.7</v>
       </c>
       <c r="N8" s="31" t="inlineStr">
         <is>
-          <t>Saatte ~14 Boy</t>
+          <t>Saatte ~49 Boy</t>
         </is>
       </c>
       <c r="O8" s="48" t="n">
-        <v>0.6605369837259856</v>
+        <v>0.6026230409833272</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -4974,13 +4974,13 @@
         </is>
       </c>
       <c r="H10" s="28" t="n">
-        <v>1397</v>
+        <v>1421</v>
       </c>
       <c r="I10" s="29" t="n">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J10" s="29" t="n">
-        <v>44050</v>
+        <v>45110</v>
       </c>
       <c r="K10" s="25" t="inlineStr">
         <is>
@@ -4988,10 +4988,10 @@
         </is>
       </c>
       <c r="L10" s="26" t="n">
-        <v>73011</v>
+        <v>74736</v>
       </c>
       <c r="M10" s="30" t="n">
-        <v>52.3</v>
+        <v>52.6</v>
       </c>
       <c r="N10" s="31" t="inlineStr">
         <is>
@@ -4999,7 +4999,7 @@
         </is>
       </c>
       <c r="O10" s="48" t="n">
-        <v>0.3927258550196062</v>
+        <v>0.3973769590166728</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -5064,7 +5064,7 @@
         </is>
       </c>
       <c r="O11" s="49" t="n">
-        <v>0.5155254807276436</v>
+        <v>0.511342853573251</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -5104,13 +5104,13 @@
         </is>
       </c>
       <c r="H12" s="28" t="n">
-        <v>911</v>
+        <v>935</v>
       </c>
       <c r="I12" s="29" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J12" s="29" t="n">
-        <v>16017</v>
+        <v>16287</v>
       </c>
       <c r="K12" s="25" t="inlineStr">
         <is>
@@ -5118,18 +5118,18 @@
         </is>
       </c>
       <c r="L12" s="26" t="n">
-        <v>61854.8</v>
+        <v>62932.8</v>
       </c>
       <c r="M12" s="30" t="n">
-        <v>67.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="N12" s="31" t="inlineStr">
         <is>
-          <t>Saatte ~18 Boy</t>
+          <t>Saatte ~17 Boy</t>
         </is>
       </c>
       <c r="O12" s="48" t="n">
-        <v>0.4693443650419077</v>
+        <v>0.4736497480954754</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -5259,7 +5259,7 @@
         </is>
       </c>
       <c r="O14" s="48" t="n">
-        <v>0.2251571588038306</v>
+        <v>0.2216605454177391</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -5364,13 +5364,13 @@
         </is>
       </c>
       <c r="H16" s="28" t="n">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="I16" s="29" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J16" s="29" t="n">
-        <v>7205</v>
+        <v>7535</v>
       </c>
       <c r="K16" s="25" t="inlineStr">
         <is>
@@ -5378,10 +5378,10 @@
         </is>
       </c>
       <c r="L16" s="26" t="n">
-        <v>30621.25</v>
+        <v>32023.75</v>
       </c>
       <c r="M16" s="30" t="n">
-        <v>92.5</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="N16" s="31" t="inlineStr">
         <is>
@@ -5429,13 +5429,13 @@
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="J17" s="15" t="n">
-        <v>7168</v>
+        <v>7938</v>
       </c>
       <c r="K17" s="10" t="inlineStr">
         <is>
@@ -5443,10 +5443,10 @@
         </is>
       </c>
       <c r="L17" s="11" t="n">
-        <v>27487</v>
+        <v>30342</v>
       </c>
       <c r="M17" s="16" t="n">
-        <v>107.8</v>
+        <v>108.8</v>
       </c>
       <c r="N17" s="17" t="inlineStr">
         <is>
@@ -5525,27 +5525,27 @@
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>KT100-220x24-ANT</t>
+          <t>140 mm KASA</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Deck / WPC Zemin</t>
+          <t>Kasa Profili</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>3.00 Metre</t>
+          <t>2.15 Metre (215 cm)</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>220 x 24 mm</t>
+          <t>140 x 36 mm</t>
         </is>
       </c>
       <c r="E19" s="45" t="inlineStr">
         <is>
-          <t>Hat 107</t>
+          <t>Hat 102</t>
         </is>
       </c>
       <c r="F19" s="18" t="inlineStr">
@@ -5553,64 +5553,64 @@
           <t>Tek Göz (1 Kafa)</t>
         </is>
       </c>
-      <c r="G19" s="12" t="inlineStr">
-        <is>
-          <t>ANA ROTA</t>
+      <c r="G19" s="20" t="inlineStr">
+        <is>
+          <t>YEDEK ROTA 2</t>
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>205.7</v>
+        <v>302</v>
       </c>
       <c r="I19" s="15" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="J19" s="15" t="n">
-        <v>1712</v>
+        <v>3301</v>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>10.33 kg/boy</t>
+          <t>4.95 kg/boy</t>
         </is>
       </c>
       <c r="L19" s="11" t="n">
-        <v>17678</v>
+        <v>18238</v>
       </c>
       <c r="M19" s="16" t="n">
-        <v>85.90000000000001</v>
+        <v>60.4</v>
       </c>
       <c r="N19" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~8 Boy</t>
+          <t>Saatte ~11 Boy</t>
         </is>
       </c>
       <c r="O19" s="49" t="n">
-        <v>1</v>
+        <v>0.1054859886058012</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>140 mm KASA</t>
+          <t>KT100-220x24-ANT</t>
         </is>
       </c>
       <c r="B20" s="24" t="inlineStr">
         <is>
-          <t>Kasa Profili</t>
+          <t>Deck / WPC Zemin</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>2.15 Metre (215 cm)</t>
+          <t>3.00 Metre</t>
         </is>
       </c>
       <c r="D20" s="24" t="inlineStr">
         <is>
-          <t>140 x 36 mm</t>
+          <t>220 x 24 mm</t>
         </is>
       </c>
       <c r="E20" s="43" t="inlineStr">
         <is>
-          <t>Hat 102</t>
+          <t>Hat 107</t>
         </is>
       </c>
       <c r="F20" s="32" t="inlineStr">
@@ -5618,38 +5618,38 @@
           <t>Tek Göz (1 Kafa)</t>
         </is>
       </c>
-      <c r="G20" s="34" t="inlineStr">
-        <is>
-          <t>YEDEK ROTA 2</t>
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>ANA ROTA</t>
         </is>
       </c>
       <c r="H20" s="28" t="n">
-        <v>281</v>
+        <v>205.7</v>
       </c>
       <c r="I20" s="29" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="J20" s="29" t="n">
-        <v>3136</v>
+        <v>1712</v>
       </c>
       <c r="K20" s="25" t="inlineStr">
         <is>
-          <t>4.95 kg/boy</t>
+          <t>10.33 kg/boy</t>
         </is>
       </c>
       <c r="L20" s="26" t="n">
-        <v>17370</v>
+        <v>17678</v>
       </c>
       <c r="M20" s="30" t="n">
-        <v>61.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="N20" s="31" t="inlineStr">
         <is>
-          <t>Saatte ~11 Boy</t>
+          <t>Saatte ~8 Boy</t>
         </is>
       </c>
       <c r="O20" s="48" t="n">
-        <v>0.1020504083191352</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
@@ -6364,7 +6364,7 @@
         </is>
       </c>
       <c r="O31" s="49" t="n">
-        <v>0.01171149544412049</v>
+        <v>0.01166411417024152</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
@@ -6689,7 +6689,7 @@
         </is>
       </c>
       <c r="O36" s="48" t="n">
-        <v>0.008048880794312908</v>
+        <v>0.007923884438532057</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
@@ -6754,7 +6754,7 @@
         </is>
       </c>
       <c r="O37" s="49" t="n">
-        <v>0.008748780254617582</v>
+        <v>0.008677798533579995</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
@@ -6884,7 +6884,7 @@
         </is>
       </c>
       <c r="O39" s="49" t="n">
-        <v>0.00638137397583121</v>
+        <v>0.006329599797693648</v>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
@@ -6949,7 +6949,7 @@
         </is>
       </c>
       <c r="O40" s="48" t="n">
-        <v>0.002559889714561856</v>
+        <v>0.00254953315196536</v>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
@@ -7014,7 +7014,7 @@
         </is>
       </c>
       <c r="O41" s="49" t="n">
-        <v>0.004206568356735797</v>
+        <v>0.00414124179415252</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
@@ -7160,15 +7160,15 @@
       <c r="F44" s="40" t="n"/>
       <c r="G44" s="40" t="n"/>
       <c r="H44" s="42" t="n">
-        <v>15736.4</v>
+        <v>15911.4</v>
       </c>
       <c r="I44" s="40" t="n"/>
       <c r="J44" s="41" t="n">
-        <v>379264</v>
+        <v>383119</v>
       </c>
       <c r="K44" s="40" t="n"/>
       <c r="L44" s="41" t="n">
-        <v>1239963.98</v>
+        <v>1252309.48</v>
       </c>
       <c r="M44" s="40" t="n"/>
       <c r="N44" s="40" t="n"/>
@@ -7469,30 +7469,30 @@
         </is>
       </c>
       <c r="E7" s="14" t="n">
-        <v>911</v>
+        <v>935</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>61854.8</v>
+        <v>62932.8</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>16017</v>
+        <v>16287</v>
       </c>
       <c r="I7" s="16" t="n">
-        <v>67.90000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="J7" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~18 Boy</t>
+          <t>Saatte ~17 Boy</t>
         </is>
       </c>
       <c r="K7" s="14" t="n">
         <v>69.5</v>
       </c>
       <c r="L7" s="19" t="n">
-        <v>0.9769784172661872</v>
+        <v>0.9683453237410071</v>
       </c>
       <c r="M7" s="8" t="inlineStr">
         <is>
@@ -7522,19 +7522,19 @@
         </is>
       </c>
       <c r="E8" s="28" t="n">
-        <v>281</v>
+        <v>302</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G8" s="26" t="n">
-        <v>17370</v>
+        <v>18238</v>
       </c>
       <c r="H8" s="29" t="n">
-        <v>3136</v>
+        <v>3301</v>
       </c>
       <c r="I8" s="30" t="n">
-        <v>61.8</v>
+        <v>60.4</v>
       </c>
       <c r="J8" s="31" t="inlineStr">
         <is>
@@ -7545,7 +7545,7 @@
         <v>51.8</v>
       </c>
       <c r="L8" s="33" t="n">
-        <v>1.193050193050193</v>
+        <v>1.166023166023166</v>
       </c>
       <c r="M8" s="24" t="inlineStr">
         <is>
@@ -7628,19 +7628,19 @@
         </is>
       </c>
       <c r="E10" s="28" t="n">
-        <v>1561.3</v>
+        <v>1585.3</v>
       </c>
       <c r="F10" s="29" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>112430</v>
+        <v>114247</v>
       </c>
       <c r="H10" s="29" t="n">
-        <v>22015</v>
+        <v>22355</v>
       </c>
       <c r="I10" s="30" t="n">
-        <v>72</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="J10" s="31" t="inlineStr">
         <is>
@@ -7651,7 +7651,7 @@
         <v>74.09999999999999</v>
       </c>
       <c r="L10" s="33" t="n">
-        <v>0.97165991902834</v>
+        <v>0.9730094466936572</v>
       </c>
       <c r="M10" s="24" t="inlineStr">
         <is>
@@ -8158,19 +8158,19 @@
         </is>
       </c>
       <c r="E20" s="55" t="n">
-        <v>1325</v>
+        <v>1349</v>
       </c>
       <c r="F20" s="56" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G20" s="57" t="n">
-        <v>68720</v>
+        <v>70445</v>
       </c>
       <c r="H20" s="56" t="n">
-        <v>41310</v>
+        <v>42370</v>
       </c>
       <c r="I20" s="58" t="n">
-        <v>51.9</v>
+        <v>52.2</v>
       </c>
       <c r="J20" s="59" t="inlineStr">
         <is>
@@ -8181,7 +8181,7 @@
         <v>53.1</v>
       </c>
       <c r="L20" s="60" t="n">
-        <v>0.9774011299435028</v>
+        <v>0.9830508474576272</v>
       </c>
       <c r="M20" s="61" t="inlineStr">
         <is>
@@ -8264,19 +8264,19 @@
         </is>
       </c>
       <c r="E22" s="55" t="n">
-        <v>1402.2</v>
+        <v>1420.2</v>
       </c>
       <c r="F22" s="56" t="n">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G22" s="57" t="n">
-        <v>105156.75</v>
+        <v>105596.75</v>
       </c>
       <c r="H22" s="56" t="n">
-        <v>70115</v>
+        <v>70470</v>
       </c>
       <c r="I22" s="58" t="n">
-        <v>75</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="J22" s="59" t="inlineStr">
         <is>
@@ -8287,7 +8287,7 @@
         <v>73.59999999999999</v>
       </c>
       <c r="L22" s="60" t="n">
-        <v>1.019021739130435</v>
+        <v>1.010869565217391</v>
       </c>
       <c r="M22" s="61" t="inlineStr">
         <is>
@@ -8688,19 +8688,19 @@
         </is>
       </c>
       <c r="E30" s="28" t="n">
-        <v>1198.5</v>
+        <v>1204.5</v>
       </c>
       <c r="F30" s="29" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G30" s="26" t="n">
-        <v>118792.08</v>
+        <v>119746.08</v>
       </c>
       <c r="H30" s="29" t="n">
-        <v>24904</v>
+        <v>25104</v>
       </c>
       <c r="I30" s="30" t="n">
-        <v>99.09999999999999</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="J30" s="31" t="inlineStr">
         <is>
@@ -8711,7 +8711,7 @@
         <v>187.9</v>
       </c>
       <c r="L30" s="38" t="n">
-        <v>0.5274081958488557</v>
+        <v>0.5290047897817989</v>
       </c>
       <c r="M30" s="24" t="inlineStr">
         <is>
@@ -9006,19 +9006,19 @@
         </is>
       </c>
       <c r="E36" s="28" t="n">
-        <v>331</v>
+        <v>341</v>
       </c>
       <c r="F36" s="29" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G36" s="26" t="n">
-        <v>30621.25</v>
+        <v>32023.75</v>
       </c>
       <c r="H36" s="29" t="n">
-        <v>7205</v>
+        <v>7535</v>
       </c>
       <c r="I36" s="30" t="n">
-        <v>92.5</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="J36" s="31" t="inlineStr">
         <is>
@@ -9029,7 +9029,7 @@
         <v>131.5</v>
       </c>
       <c r="L36" s="38" t="n">
-        <v>0.7034220532319392</v>
+        <v>0.7140684410646387</v>
       </c>
       <c r="M36" s="24" t="inlineStr">
         <is>
@@ -9165,19 +9165,19 @@
         </is>
       </c>
       <c r="E39" s="55" t="n">
-        <v>1502.4</v>
+        <v>1526.4</v>
       </c>
       <c r="F39" s="56" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G39" s="57" t="n">
-        <v>144935.32</v>
+        <v>146141.32</v>
       </c>
       <c r="H39" s="56" t="n">
-        <v>42511</v>
+        <v>42876</v>
       </c>
       <c r="I39" s="58" t="n">
-        <v>96.5</v>
+        <v>95.7</v>
       </c>
       <c r="J39" s="59" t="inlineStr">
         <is>
@@ -9188,7 +9188,7 @@
         <v>99.2</v>
       </c>
       <c r="L39" s="60" t="n">
-        <v>0.9727822580645161</v>
+        <v>0.9647177419354839</v>
       </c>
       <c r="M39" s="61" t="inlineStr">
         <is>
@@ -9377,19 +9377,19 @@
         </is>
       </c>
       <c r="E43" s="14" t="n">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="F43" s="15" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G43" s="11" t="n">
-        <v>27487</v>
+        <v>30342</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>7168</v>
+        <v>7938</v>
       </c>
       <c r="I43" s="16" t="n">
-        <v>107.8</v>
+        <v>108.8</v>
       </c>
       <c r="J43" s="17" t="inlineStr">
         <is>
@@ -9400,7 +9400,7 @@
         <v>96.09999999999999</v>
       </c>
       <c r="L43" s="19" t="n">
-        <v>1.121748178980229</v>
+        <v>1.132154006243496</v>
       </c>
       <c r="M43" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(levha): saat girilen donemden net seri uretim hizi hesaplandi (40-43 plaka/saat = 1000 plaka/gun = 500 kapi)
</commit_message>
<xml_diff>
--- a/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
+++ b/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
@@ -868,7 +868,7 @@
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>Fiili Hız (Saatte ~X Boy)</t>
+          <t>Fiili Hız (Saatte ~X Boy/Plaka)</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="O4" s="6" t="inlineStr">
         <is>
-          <t>Standart Hız (Saatte ~X Boy)</t>
+          <t>Standart Hız (Saatte ~X Boy/Plaka)</t>
         </is>
       </c>
       <c r="P4" s="6" t="inlineStr">
@@ -1380,32 +1380,32 @@
         </is>
       </c>
       <c r="I9" s="14" t="n">
-        <v>1218.5</v>
+        <v>622.6096835790281</v>
       </c>
       <c r="J9" s="15" t="n">
         <v>84</v>
       </c>
       <c r="K9" s="16" t="n">
-        <v>100.7</v>
+        <v>203.9</v>
       </c>
       <c r="L9" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~21 Plaka</t>
+          <t>Saatte ~43 Plaka</t>
         </is>
       </c>
       <c r="M9" s="11" t="n">
-        <v>2416.8</v>
+        <v>4893.6</v>
       </c>
       <c r="N9" s="14" t="n">
-        <v>187.9</v>
+        <v>190</v>
       </c>
       <c r="O9" s="18" t="inlineStr">
         <is>
-          <t>Saatte ~39 Plaka</t>
-        </is>
-      </c>
-      <c r="P9" s="39" t="n">
-        <v>0.536</v>
+          <t>Saatte ~40 Plaka</t>
+        </is>
+      </c>
+      <c r="P9" s="19" t="n">
+        <v>1.073</v>
       </c>
       <c r="Q9" s="23" t="inlineStr">
         <is>
@@ -1590,32 +1590,32 @@
         </is>
       </c>
       <c r="I11" s="14" t="n">
-        <v>350.5</v>
+        <v>235.1702808249805</v>
       </c>
       <c r="J11" s="15" t="n">
         <v>37</v>
       </c>
       <c r="K11" s="16" t="n">
-        <v>113.5</v>
+        <v>165.8</v>
       </c>
       <c r="L11" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~27 Plaka</t>
+          <t>Saatte ~39 Plaka</t>
         </is>
       </c>
       <c r="M11" s="11" t="n">
-        <v>2724</v>
+        <v>3979.2</v>
       </c>
       <c r="N11" s="14" t="n">
-        <v>145.5</v>
+        <v>190</v>
       </c>
       <c r="O11" s="18" t="inlineStr">
         <is>
-          <t>Saatte ~34 Plaka</t>
-        </is>
-      </c>
-      <c r="P11" s="39" t="n">
-        <v>0.78</v>
+          <t>Saatte ~45 Plaka</t>
+        </is>
+      </c>
+      <c r="P11" s="19" t="n">
+        <v>0.873</v>
       </c>
       <c r="Q11" s="23" t="inlineStr">
         <is>
@@ -1698,32 +1698,32 @@
         </is>
       </c>
       <c r="I12" s="29" t="n">
-        <v>343</v>
+        <v>187.6562562708018</v>
       </c>
       <c r="J12" s="30" t="n">
         <v>31</v>
       </c>
       <c r="K12" s="31" t="n">
-        <v>95.09999999999999</v>
+        <v>174</v>
       </c>
       <c r="L12" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~22 Plaka</t>
+          <t>Saatte ~41 Plaka</t>
         </is>
       </c>
       <c r="M12" s="27" t="n">
-        <v>2282.4</v>
+        <v>4176</v>
       </c>
       <c r="N12" s="29" t="n">
-        <v>131.5</v>
+        <v>190</v>
       </c>
       <c r="O12" s="33" t="inlineStr">
         <is>
-          <t>Saatte ~31 Plaka</t>
-        </is>
-      </c>
-      <c r="P12" s="40" t="n">
-        <v>0.723</v>
+          <t>Saatte ~45 Plaka</t>
+        </is>
+      </c>
+      <c r="P12" s="34" t="n">
+        <v>0.9159999999999999</v>
       </c>
       <c r="Q12" s="38" t="inlineStr">
         <is>
@@ -1914,32 +1914,32 @@
         </is>
       </c>
       <c r="I14" s="29" t="n">
-        <v>260</v>
+        <v>173.7487454529077</v>
       </c>
       <c r="J14" s="30" t="n">
         <v>30</v>
       </c>
       <c r="K14" s="31" t="n">
-        <v>123.3</v>
+        <v>178.7</v>
       </c>
       <c r="L14" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~28 Plaka</t>
+          <t>Saatte ~40 Plaka</t>
         </is>
       </c>
       <c r="M14" s="27" t="n">
-        <v>2959.2</v>
+        <v>4288.8</v>
       </c>
       <c r="N14" s="29" t="n">
-        <v>148.4</v>
+        <v>190</v>
       </c>
       <c r="O14" s="33" t="inlineStr">
         <is>
-          <t>Saatte ~34 Plaka</t>
+          <t>Saatte ~43 Plaka</t>
         </is>
       </c>
       <c r="P14" s="34" t="n">
-        <v>0.831</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="Q14" s="38" t="inlineStr">
         <is>
@@ -2022,32 +2022,32 @@
         </is>
       </c>
       <c r="I15" s="14" t="n">
-        <v>193</v>
+        <v>114.2245721724266</v>
       </c>
       <c r="J15" s="15" t="n">
         <v>22</v>
       </c>
       <c r="K15" s="16" t="n">
-        <v>95.2</v>
+        <v>159.9</v>
       </c>
       <c r="L15" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~20 Plaka</t>
+          <t>Saatte ~34 Plaka</t>
         </is>
       </c>
       <c r="M15" s="11" t="n">
-        <v>2284.8</v>
+        <v>3837.6</v>
       </c>
       <c r="N15" s="14" t="n">
-        <v>116.2</v>
+        <v>190</v>
       </c>
       <c r="O15" s="18" t="inlineStr">
         <is>
-          <t>Saatte ~24 Plaka</t>
+          <t>Saatte ~40 Plaka</t>
         </is>
       </c>
       <c r="P15" s="19" t="n">
-        <v>0.8190000000000001</v>
+        <v>0.8420000000000001</v>
       </c>
       <c r="Q15" s="23" t="inlineStr">
         <is>
@@ -2664,32 +2664,32 @@
         </is>
       </c>
       <c r="I21" s="14" t="n">
-        <v>69</v>
+        <v>48.79255891118007</v>
       </c>
       <c r="J21" s="15" t="n">
         <v>9</v>
       </c>
       <c r="K21" s="16" t="n">
-        <v>132.2</v>
+        <v>187.5</v>
       </c>
       <c r="L21" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~31 Plaka</t>
+          <t>Saatte ~44 Plaka</t>
         </is>
       </c>
       <c r="M21" s="11" t="n">
-        <v>3172.8</v>
+        <v>4500</v>
       </c>
       <c r="N21" s="14" t="n">
-        <v>118.6</v>
+        <v>190</v>
       </c>
       <c r="O21" s="18" t="inlineStr">
         <is>
-          <t>Saatte ~28 Plaka</t>
+          <t>Saatte ~45 Plaka</t>
         </is>
       </c>
       <c r="P21" s="19" t="n">
-        <v>1.115</v>
+        <v>0.987</v>
       </c>
       <c r="Q21" s="23" t="inlineStr">
         <is>
@@ -2880,32 +2880,32 @@
         </is>
       </c>
       <c r="I23" s="14" t="n">
-        <v>106</v>
+        <v>57.25702552864577</v>
       </c>
       <c r="J23" s="15" t="n">
         <v>13</v>
       </c>
       <c r="K23" s="16" t="n">
-        <v>72.5</v>
+        <v>131.6</v>
       </c>
       <c r="L23" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~17 Plaka</t>
+          <t>Saatte ~30 Plaka</t>
         </is>
       </c>
       <c r="M23" s="11" t="n">
-        <v>1740</v>
+        <v>3158.4</v>
       </c>
       <c r="N23" s="14" t="n">
-        <v>113.1</v>
+        <v>190</v>
       </c>
       <c r="O23" s="18" t="inlineStr">
         <is>
-          <t>Saatte ~26 Plaka</t>
+          <t>Saatte ~44 Plaka</t>
         </is>
       </c>
       <c r="P23" s="39" t="n">
-        <v>0.6409999999999999</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="Q23" s="23" t="inlineStr">
         <is>
@@ -2988,32 +2988,32 @@
         </is>
       </c>
       <c r="I24" s="29" t="n">
-        <v>57.5</v>
+        <v>38.03440860215053</v>
       </c>
       <c r="J24" s="30" t="n">
         <v>8</v>
       </c>
       <c r="K24" s="31" t="n">
-        <v>104.7</v>
+        <v>185.6</v>
       </c>
       <c r="L24" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~23 Plaka</t>
+          <t>Saatte ~40 Plaka</t>
         </is>
       </c>
       <c r="M24" s="27" t="n">
-        <v>2512.8</v>
+        <v>4454.4</v>
       </c>
       <c r="N24" s="29" t="n">
-        <v>144.9</v>
+        <v>190</v>
       </c>
       <c r="O24" s="33" t="inlineStr">
         <is>
-          <t>Saatte ~31 Plaka</t>
-        </is>
-      </c>
-      <c r="P24" s="40" t="n">
-        <v>0.723</v>
+          <t>Saatte ~41 Plaka</t>
+        </is>
+      </c>
+      <c r="P24" s="34" t="n">
+        <v>0.977</v>
       </c>
       <c r="Q24" s="38" t="inlineStr">
         <is>
@@ -3096,32 +3096,32 @@
         </is>
       </c>
       <c r="I25" s="14" t="n">
-        <v>78</v>
+        <v>41.52884989747753</v>
       </c>
       <c r="J25" s="15" t="n">
         <v>8</v>
       </c>
       <c r="K25" s="16" t="n">
-        <v>71.90000000000001</v>
+        <v>35</v>
       </c>
       <c r="L25" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~15 Plaka</t>
+          <t>Saatte ~7 Plaka</t>
         </is>
       </c>
       <c r="M25" s="11" t="n">
-        <v>1725.6</v>
+        <v>840</v>
       </c>
       <c r="N25" s="14" t="n">
-        <v>111.8</v>
+        <v>190</v>
       </c>
       <c r="O25" s="18" t="inlineStr">
         <is>
-          <t>Saatte ~23 Plaka</t>
+          <t>Saatte ~40 Plaka</t>
         </is>
       </c>
       <c r="P25" s="39" t="n">
-        <v>0.643</v>
+        <v>0.184</v>
       </c>
       <c r="Q25" s="23" t="inlineStr">
         <is>
@@ -3204,32 +3204,32 @@
         </is>
       </c>
       <c r="I26" s="29" t="n">
-        <v>72.5</v>
+        <v>31.97761876040141</v>
       </c>
       <c r="J26" s="30" t="n">
         <v>7</v>
       </c>
       <c r="K26" s="31" t="n">
-        <v>53.1</v>
+        <v>95.8</v>
       </c>
       <c r="L26" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~11 Plaka</t>
+          <t>Saatte ~20 Plaka</t>
         </is>
       </c>
       <c r="M26" s="27" t="n">
-        <v>1274.4</v>
+        <v>2299.2</v>
       </c>
       <c r="N26" s="29" t="n">
-        <v>79.2</v>
+        <v>190</v>
       </c>
       <c r="O26" s="33" t="inlineStr">
         <is>
-          <t>Saatte ~16 Plaka</t>
+          <t>Saatte ~40 Plaka</t>
         </is>
       </c>
       <c r="P26" s="40" t="n">
-        <v>0.67</v>
+        <v>0.504</v>
       </c>
       <c r="Q26" s="38" t="inlineStr">
         <is>
@@ -3318,26 +3318,26 @@
         <v>3</v>
       </c>
       <c r="K27" s="16" t="n">
-        <v>198.2</v>
+        <v>134.1</v>
       </c>
       <c r="L27" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~41 Plaka</t>
+          <t>Saatte ~28 Plaka</t>
         </is>
       </c>
       <c r="M27" s="11" t="n">
-        <v>4756.8</v>
+        <v>3218.4</v>
       </c>
       <c r="N27" s="14" t="n">
-        <v>273.6</v>
+        <v>190</v>
       </c>
       <c r="O27" s="18" t="inlineStr">
         <is>
-          <t>Saatte ~57 Plaka</t>
+          <t>Saatte ~40 Plaka</t>
         </is>
       </c>
       <c r="P27" s="39" t="n">
-        <v>0.7240000000000001</v>
+        <v>0.706</v>
       </c>
       <c r="Q27" s="23" t="inlineStr">
         <is>
@@ -3720,7 +3720,7 @@
       <c r="G31" s="42" t="n"/>
       <c r="H31" s="42" t="n"/>
       <c r="I31" s="44" t="n">
-        <v>11092.7</v>
+        <v>9895.700000000003</v>
       </c>
       <c r="J31" s="42" t="n"/>
       <c r="K31" s="42" t="n"/>
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="D13" s="14" t="n">
-        <v>2762.5</v>
+        <v>1565.5</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>252</v>
@@ -4296,7 +4296,7 @@
         <v>280733.6800000001</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>101.6</v>
+        <v>179.3</v>
       </c>
       <c r="H13" s="48" t="n">
         <v>11</v>
@@ -4326,7 +4326,7 @@
       <c r="B14" s="42" t="n"/>
       <c r="C14" s="42" t="n"/>
       <c r="D14" s="44" t="n">
-        <v>16095.4</v>
+        <v>14898.4</v>
       </c>
       <c r="E14" s="43" t="n">
         <v>1480</v>
@@ -4335,7 +4335,7 @@
         <v>1266753.58</v>
       </c>
       <c r="G14" s="44" t="n">
-        <v>78.7</v>
+        <v>85</v>
       </c>
       <c r="H14" s="42" t="n"/>
       <c r="I14" s="42" t="n"/>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>Fiili Hız (Saatte ~X Boy)</t>
+          <t>Fiili Hız (Saatte ~X Boy/Plaka)</t>
         </is>
       </c>
       <c r="O3" s="6" t="inlineStr">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H6" s="29" t="n">
-        <v>1218.5</v>
+        <v>622.6096835790281</v>
       </c>
       <c r="I6" s="30" t="n">
         <v>84</v>
@@ -4652,11 +4652,11 @@
         <v>122751.18</v>
       </c>
       <c r="M6" s="31" t="n">
-        <v>100.7</v>
+        <v>197.2</v>
       </c>
       <c r="N6" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~21 Plaka</t>
+          <t>Saatte ~41 Plaka</t>
         </is>
       </c>
       <c r="O6" s="50" t="n">
@@ -5090,7 +5090,7 @@
         </is>
       </c>
       <c r="H13" s="14" t="n">
-        <v>350.5</v>
+        <v>235.1702808249805</v>
       </c>
       <c r="I13" s="15" t="n">
         <v>37</v>
@@ -5107,11 +5107,11 @@
         <v>39775.75</v>
       </c>
       <c r="M13" s="16" t="n">
-        <v>113.5</v>
+        <v>169.1</v>
       </c>
       <c r="N13" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~27 Plaka</t>
+          <t>Saatte ~40 Plaka</t>
         </is>
       </c>
       <c r="O13" s="51" t="n">
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="H15" s="14" t="n">
-        <v>343</v>
+        <v>187.6562562708018</v>
       </c>
       <c r="I15" s="15" t="n">
         <v>31</v>
@@ -5237,11 +5237,11 @@
         <v>32618.75</v>
       </c>
       <c r="M15" s="16" t="n">
-        <v>95.09999999999999</v>
+        <v>173.8</v>
       </c>
       <c r="N15" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~22 Plaka</t>
+          <t>Saatte ~41 Plaka</t>
         </is>
       </c>
       <c r="O15" s="51" t="n">
@@ -5350,7 +5350,7 @@
         </is>
       </c>
       <c r="H17" s="14" t="n">
-        <v>260</v>
+        <v>173.7487454529077</v>
       </c>
       <c r="I17" s="15" t="n">
         <v>30</v>
@@ -5367,11 +5367,11 @@
         <v>32060.7</v>
       </c>
       <c r="M17" s="16" t="n">
-        <v>123.3</v>
+        <v>184.5</v>
       </c>
       <c r="N17" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~28 Plaka</t>
+          <t>Saatte ~42 Plaka</t>
         </is>
       </c>
       <c r="O17" s="51" t="n">
@@ -5480,7 +5480,7 @@
         </is>
       </c>
       <c r="H19" s="14" t="n">
-        <v>193</v>
+        <v>114.2245721724266</v>
       </c>
       <c r="I19" s="15" t="n">
         <v>22</v>
@@ -5497,11 +5497,11 @@
         <v>18364.5</v>
       </c>
       <c r="M19" s="16" t="n">
-        <v>95.2</v>
+        <v>160.8</v>
       </c>
       <c r="N19" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~20 Plaka</t>
+          <t>Saatte ~34 Plaka</t>
         </is>
       </c>
       <c r="O19" s="51" t="n">
@@ -5870,7 +5870,7 @@
         </is>
       </c>
       <c r="H25" s="14" t="n">
-        <v>69</v>
+        <v>48.79255891118007</v>
       </c>
       <c r="I25" s="15" t="n">
         <v>9</v>
@@ -5887,11 +5887,11 @@
         <v>9124.75</v>
       </c>
       <c r="M25" s="16" t="n">
-        <v>132.2</v>
+        <v>187</v>
       </c>
       <c r="N25" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~31 Plaka</t>
+          <t>Saatte ~44 Plaka</t>
         </is>
       </c>
       <c r="O25" s="51" t="n">
@@ -6000,7 +6000,7 @@
         </is>
       </c>
       <c r="H27" s="14" t="n">
-        <v>106</v>
+        <v>57.25702552864577</v>
       </c>
       <c r="I27" s="15" t="n">
         <v>13</v>
@@ -6017,11 +6017,11 @@
         <v>7690.08</v>
       </c>
       <c r="M27" s="16" t="n">
-        <v>72.5</v>
+        <v>134.3</v>
       </c>
       <c r="N27" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~17 Plaka</t>
+          <t>Saatte ~31 Plaka</t>
         </is>
       </c>
       <c r="O27" s="51" t="n">
@@ -6065,7 +6065,7 @@
         </is>
       </c>
       <c r="H28" s="29" t="n">
-        <v>57.5</v>
+        <v>38.03440860215053</v>
       </c>
       <c r="I28" s="30" t="n">
         <v>8</v>
@@ -6082,11 +6082,11 @@
         <v>6018.08</v>
       </c>
       <c r="M28" s="31" t="n">
-        <v>104.7</v>
+        <v>158.2</v>
       </c>
       <c r="N28" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~23 Plaka</t>
+          <t>Saatte ~34 Plaka</t>
         </is>
       </c>
       <c r="O28" s="50" t="n">
@@ -6130,7 +6130,7 @@
         </is>
       </c>
       <c r="H29" s="14" t="n">
-        <v>78</v>
+        <v>41.52884989747753</v>
       </c>
       <c r="I29" s="15" t="n">
         <v>8</v>
@@ -6147,11 +6147,11 @@
         <v>5609.52</v>
       </c>
       <c r="M29" s="16" t="n">
-        <v>71.90000000000001</v>
+        <v>135.1</v>
       </c>
       <c r="N29" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~15 Plaka</t>
+          <t>Saatte ~28 Plaka</t>
         </is>
       </c>
       <c r="O29" s="51" t="n">
@@ -6195,7 +6195,7 @@
         </is>
       </c>
       <c r="H30" s="29" t="n">
-        <v>72.5</v>
+        <v>31.97761876040141</v>
       </c>
       <c r="I30" s="30" t="n">
         <v>7</v>
@@ -6212,11 +6212,11 @@
         <v>3846.37</v>
       </c>
       <c r="M30" s="31" t="n">
-        <v>53.1</v>
+        <v>120.3</v>
       </c>
       <c r="N30" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~11 Plaka</t>
+          <t>Saatte ~25 Plaka</t>
         </is>
       </c>
       <c r="O30" s="50" t="n">
@@ -7081,7 +7081,7 @@
       <c r="F44" s="42" t="n"/>
       <c r="G44" s="42" t="n"/>
       <c r="H44" s="44" t="n">
-        <v>16095.4</v>
+        <v>14898.4</v>
       </c>
       <c r="I44" s="42" t="n"/>
       <c r="J44" s="43" t="n">
@@ -8344,7 +8344,7 @@
         </is>
       </c>
       <c r="E25" s="14" t="n">
-        <v>78</v>
+        <v>41.52884989747753</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>8</v>
@@ -8356,18 +8356,18 @@
         <v>1176</v>
       </c>
       <c r="I25" s="16" t="n">
-        <v>71.90000000000001</v>
+        <v>135.1</v>
       </c>
       <c r="J25" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~15 Plaka</t>
+          <t>Saatte ~28 Plaka</t>
         </is>
       </c>
       <c r="K25" s="14" t="n">
-        <v>111.8</v>
+        <v>190</v>
       </c>
       <c r="L25" s="39" t="n">
-        <v>0.6431127012522362</v>
+        <v>0.7110526315789474</v>
       </c>
       <c r="M25" s="8" t="inlineStr">
         <is>
@@ -8397,7 +8397,7 @@
         </is>
       </c>
       <c r="E26" s="29" t="n">
-        <v>57.5</v>
+        <v>38.03440860215053</v>
       </c>
       <c r="F26" s="30" t="n">
         <v>8</v>
@@ -8409,18 +8409,18 @@
         <v>1297</v>
       </c>
       <c r="I26" s="31" t="n">
-        <v>104.7</v>
+        <v>158.2</v>
       </c>
       <c r="J26" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~23 Plaka</t>
+          <t>Saatte ~34 Plaka</t>
         </is>
       </c>
       <c r="K26" s="29" t="n">
-        <v>144.9</v>
-      </c>
-      <c r="L26" s="40" t="n">
-        <v>0.722567287784679</v>
+        <v>190</v>
+      </c>
+      <c r="L26" s="34" t="n">
+        <v>0.8326315789473684</v>
       </c>
       <c r="M26" s="25" t="inlineStr">
         <is>
@@ -8450,7 +8450,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>260</v>
+        <v>173.7487454529077</v>
       </c>
       <c r="F27" s="15" t="n">
         <v>30</v>
@@ -8462,18 +8462,18 @@
         <v>7270</v>
       </c>
       <c r="I27" s="16" t="n">
-        <v>123.3</v>
+        <v>184.5</v>
       </c>
       <c r="J27" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~28 Plaka</t>
+          <t>Saatte ~42 Plaka</t>
         </is>
       </c>
       <c r="K27" s="14" t="n">
-        <v>148.4</v>
+        <v>190</v>
       </c>
       <c r="L27" s="19" t="n">
-        <v>0.8308625336927222</v>
+        <v>0.9710526315789474</v>
       </c>
       <c r="M27" s="8" t="inlineStr">
         <is>
@@ -8576,10 +8576,10 @@
         </is>
       </c>
       <c r="K29" s="14" t="n">
-        <v>273.6</v>
-      </c>
-      <c r="L29" s="39" t="n">
-        <v>0.7244152046783625</v>
+        <v>190</v>
+      </c>
+      <c r="L29" s="19" t="n">
+        <v>1.043157894736842</v>
       </c>
       <c r="M29" s="8" t="inlineStr">
         <is>
@@ -8609,7 +8609,7 @@
         </is>
       </c>
       <c r="E30" s="29" t="n">
-        <v>1218.5</v>
+        <v>622.6096835790281</v>
       </c>
       <c r="F30" s="30" t="n">
         <v>84</v>
@@ -8621,18 +8621,18 @@
         <v>25734</v>
       </c>
       <c r="I30" s="31" t="n">
-        <v>100.7</v>
+        <v>197.2</v>
       </c>
       <c r="J30" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~21 Plaka</t>
+          <t>Saatte ~41 Plaka</t>
         </is>
       </c>
       <c r="K30" s="29" t="n">
-        <v>187.9</v>
-      </c>
-      <c r="L30" s="40" t="n">
-        <v>0.5359233634912187</v>
+        <v>190</v>
+      </c>
+      <c r="L30" s="34" t="n">
+        <v>1.037894736842105</v>
       </c>
       <c r="M30" s="25" t="inlineStr">
         <is>
@@ -8662,7 +8662,7 @@
         </is>
       </c>
       <c r="E31" s="14" t="n">
-        <v>72.5</v>
+        <v>31.97761876040141</v>
       </c>
       <c r="F31" s="15" t="n">
         <v>7</v>
@@ -8674,18 +8674,18 @@
         <v>803</v>
       </c>
       <c r="I31" s="16" t="n">
-        <v>53.1</v>
+        <v>120.3</v>
       </c>
       <c r="J31" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~11 Plaka</t>
+          <t>Saatte ~25 Plaka</t>
         </is>
       </c>
       <c r="K31" s="14" t="n">
-        <v>79.2</v>
+        <v>190</v>
       </c>
       <c r="L31" s="39" t="n">
-        <v>0.6704545454545454</v>
+        <v>0.6331578947368421</v>
       </c>
       <c r="M31" s="8" t="inlineStr">
         <is>
@@ -8874,7 +8874,7 @@
         </is>
       </c>
       <c r="E35" s="14" t="n">
-        <v>69</v>
+        <v>48.79255891118007</v>
       </c>
       <c r="F35" s="15" t="n">
         <v>9</v>
@@ -8886,18 +8886,18 @@
         <v>2147</v>
       </c>
       <c r="I35" s="16" t="n">
-        <v>132.2</v>
+        <v>187</v>
       </c>
       <c r="J35" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~31 Plaka</t>
+          <t>Saatte ~44 Plaka</t>
         </is>
       </c>
       <c r="K35" s="14" t="n">
-        <v>118.6</v>
+        <v>190</v>
       </c>
       <c r="L35" s="19" t="n">
-        <v>1.114671163575042</v>
+        <v>0.9842105263157894</v>
       </c>
       <c r="M35" s="8" t="inlineStr">
         <is>
@@ -8927,7 +8927,7 @@
         </is>
       </c>
       <c r="E36" s="29" t="n">
-        <v>343</v>
+        <v>187.6562562708018</v>
       </c>
       <c r="F36" s="30" t="n">
         <v>31</v>
@@ -8939,18 +8939,18 @@
         <v>7675</v>
       </c>
       <c r="I36" s="31" t="n">
-        <v>95.09999999999999</v>
+        <v>173.8</v>
       </c>
       <c r="J36" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~22 Plaka</t>
+          <t>Saatte ~41 Plaka</t>
         </is>
       </c>
       <c r="K36" s="29" t="n">
-        <v>131.5</v>
-      </c>
-      <c r="L36" s="40" t="n">
-        <v>0.7231939163498099</v>
+        <v>190</v>
+      </c>
+      <c r="L36" s="34" t="n">
+        <v>0.9147368421052632</v>
       </c>
       <c r="M36" s="25" t="inlineStr">
         <is>
@@ -9351,7 +9351,7 @@
         </is>
       </c>
       <c r="E44" s="29" t="n">
-        <v>106</v>
+        <v>57.25702552864577</v>
       </c>
       <c r="F44" s="30" t="n">
         <v>13</v>
@@ -9363,18 +9363,18 @@
         <v>1776</v>
       </c>
       <c r="I44" s="31" t="n">
-        <v>72.5</v>
+        <v>134.3</v>
       </c>
       <c r="J44" s="32" t="inlineStr">
         <is>
-          <t>Saatte ~17 Plaka</t>
+          <t>Saatte ~31 Plaka</t>
         </is>
       </c>
       <c r="K44" s="29" t="n">
-        <v>113.1</v>
+        <v>190</v>
       </c>
       <c r="L44" s="40" t="n">
-        <v>0.641025641025641</v>
+        <v>0.7068421052631579</v>
       </c>
       <c r="M44" s="25" t="inlineStr">
         <is>
@@ -9404,7 +9404,7 @@
         </is>
       </c>
       <c r="E45" s="14" t="n">
-        <v>350.5</v>
+        <v>235.1702808249805</v>
       </c>
       <c r="F45" s="15" t="n">
         <v>37</v>
@@ -9416,18 +9416,18 @@
         <v>9359</v>
       </c>
       <c r="I45" s="16" t="n">
-        <v>113.5</v>
+        <v>169.1</v>
       </c>
       <c r="J45" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~27 Plaka</t>
+          <t>Saatte ~40 Plaka</t>
         </is>
       </c>
       <c r="K45" s="14" t="n">
-        <v>145.5</v>
-      </c>
-      <c r="L45" s="39" t="n">
-        <v>0.7800687285223369</v>
+        <v>190</v>
+      </c>
+      <c r="L45" s="19" t="n">
+        <v>0.89</v>
       </c>
       <c r="M45" s="8" t="inlineStr">
         <is>
@@ -9510,7 +9510,7 @@
         </is>
       </c>
       <c r="E47" s="14" t="n">
-        <v>193</v>
+        <v>114.2245721724266</v>
       </c>
       <c r="F47" s="15" t="n">
         <v>22</v>
@@ -9522,18 +9522,18 @@
         <v>3850</v>
       </c>
       <c r="I47" s="16" t="n">
-        <v>95.2</v>
+        <v>160.8</v>
       </c>
       <c r="J47" s="17" t="inlineStr">
         <is>
-          <t>Saatte ~20 Plaka</t>
+          <t>Saatte ~34 Plaka</t>
         </is>
       </c>
       <c r="K47" s="14" t="n">
-        <v>116.2</v>
+        <v>190</v>
       </c>
       <c r="L47" s="19" t="n">
-        <v>0.8192771084337349</v>
+        <v>0.8463157894736842</v>
       </c>
       <c r="M47" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update static Excel with AutoFilter and SUBTOTAL
</commit_message>
<xml_diff>
--- a/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
+++ b/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
@@ -2790,19 +2790,19 @@
         </is>
       </c>
       <c r="I23" s="14" t="n">
-        <v>47.95702552864577</v>
+        <v>48.25702552864577</v>
       </c>
       <c r="J23" s="15" t="n">
         <v>13</v>
       </c>
       <c r="K23" s="16" t="n">
-        <v>167.9</v>
+        <v>166.5</v>
       </c>
       <c r="L23" s="41" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M23" s="11" t="n">
-        <v>4029.6</v>
+        <v>3996</v>
       </c>
       <c r="N23" s="14" t="n">
         <v>190</v>
@@ -2811,7 +2811,7 @@
         <v>44</v>
       </c>
       <c r="P23" s="19" t="n">
-        <v>0.884</v>
+        <v>0.8759999999999999</v>
       </c>
       <c r="Q23" s="23" t="inlineStr">
         <is>
@@ -2994,7 +2994,7 @@
         </is>
       </c>
       <c r="I25" s="14" t="n">
-        <v>37.72884989747753</v>
+        <v>38.52884989747753</v>
       </c>
       <c r="J25" s="15" t="n">
         <v>8</v>
@@ -4161,7 +4161,7 @@
         </is>
       </c>
       <c r="D13" s="14" t="n">
-        <v>1562.4</v>
+        <v>1563.5</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>253</v>
@@ -4170,7 +4170,7 @@
         <v>283404.8800000001</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>181.4</v>
+        <v>181.3</v>
       </c>
       <c r="H13" s="56" t="n">
         <v>11</v>
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="H27" s="14" t="n">
-        <v>47.95702552864577</v>
+        <v>48.25702552864577</v>
       </c>
       <c r="I27" s="15" t="n">
         <v>13</v>
@@ -5802,7 +5802,7 @@
         <v>7690.08</v>
       </c>
       <c r="M27" s="16" t="n">
-        <v>160.4</v>
+        <v>159.4</v>
       </c>
       <c r="N27" s="41" t="n">
         <v>37</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="H29" s="14" t="n">
-        <v>37.72884989747753</v>
+        <v>38.52884989747753</v>
       </c>
       <c r="I29" s="15" t="n">
         <v>8</v>
@@ -5924,7 +5924,7 @@
         <v>5609.52</v>
       </c>
       <c r="M29" s="16" t="n">
-        <v>148.7</v>
+        <v>145.6</v>
       </c>
       <c r="N29" s="41" t="n">
         <v>31</v>
@@ -8028,7 +8028,7 @@
         </is>
       </c>
       <c r="E25" s="14" t="n">
-        <v>37.72884989747753</v>
+        <v>38.52884989747753</v>
       </c>
       <c r="F25" s="15" t="n">
         <v>8</v>
@@ -8040,16 +8040,16 @@
         <v>1176</v>
       </c>
       <c r="I25" s="16" t="n">
-        <v>148.7</v>
+        <v>145.6</v>
       </c>
       <c r="J25" s="41" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="K25" s="14" t="n">
         <v>190</v>
       </c>
       <c r="L25" s="48" t="n">
-        <v>0.7826315789473683</v>
+        <v>0.7663157894736841</v>
       </c>
       <c r="M25" s="8" t="inlineStr">
         <is>
@@ -8997,7 +8997,7 @@
         </is>
       </c>
       <c r="E44" s="29" t="n">
-        <v>47.95702552864577</v>
+        <v>48.25702552864577</v>
       </c>
       <c r="F44" s="30" t="n">
         <v>13</v>
@@ -9009,7 +9009,7 @@
         <v>1776</v>
       </c>
       <c r="I44" s="31" t="n">
-        <v>160.4</v>
+        <v>159.4</v>
       </c>
       <c r="J44" s="45" t="n">
         <v>37</v>
@@ -9018,7 +9018,7 @@
         <v>190</v>
       </c>
       <c r="L44" s="34" t="n">
-        <v>0.8442105263157896</v>
+        <v>0.8389473684210526</v>
       </c>
       <c r="M44" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
COCO Levha fiili saat ve hizi Excelde 14.5 saat ve 41 plaka/sa olarak guncellendi
</commit_message>
<xml_diff>
--- a/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
+++ b/static/Ergunbas_Urun_Hat_Rotalari_ve_Kapasite_Analizi.xlsx
@@ -773,7 +773,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:X31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -3204,13 +3204,13 @@
         <v>3</v>
       </c>
       <c r="K27" s="16" t="n">
-        <v>134.1</v>
+        <v>198.2</v>
       </c>
       <c r="L27" s="41" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="M27" s="11" t="n">
-        <v>3218.4</v>
+        <v>4756.8</v>
       </c>
       <c r="N27" s="14" t="n">
         <v>190</v>
@@ -3219,7 +3219,7 @@
         <v>40</v>
       </c>
       <c r="P27" s="48" t="n">
-        <v>0.706</v>
+        <v>1.043158</v>
       </c>
       <c r="Q27" s="23" t="inlineStr">
         <is>
@@ -3635,7 +3635,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -4237,7 +4237,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O44"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -6837,7 +6837,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M48"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>

</xml_diff>